<commit_message>
Anonymize workplan sample data to Stream/Task labels
Replace domain-specific stream names, tasks, roles and milestones with neutral Stream 1–5 and Task N.M placeholders for safe sharing.

Co-authored-by: dimonix2019 <dimonix2019@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/plan_docs_export/Plan_rabot_strimy.xlsx
+++ b/plan_docs_export/Plan_rabot_strimy.xlsx
@@ -36,10 +36,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="DD.MM.YYYY"/>
-    <numFmt numFmtId="166" formatCode="DD.MM"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="DD.MM.YYYY"/>
+    <numFmt numFmtId="165" formatCode="DD.MM"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -239,7 +238,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="83">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -296,13 +295,13 @@
     <xf numFmtId="0" fontId="6" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="6" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -311,19 +310,19 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="8" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="7" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -341,7 +340,7 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -353,7 +352,7 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -365,7 +364,7 @@
     <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -377,7 +376,7 @@
     <xf numFmtId="0" fontId="2" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="2" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -389,7 +388,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -416,7 +415,7 @@
     <xf numFmtId="0" fontId="2" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -429,6 +428,42 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -949,14 +984,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>План работ по стримам — личный слой планирования (не замена Confluence)</t>
+          <t>План работ по стримам — личный слой планирования (не замена доска)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="36" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Confluence остаётся отчётной доской. Этот файл — последовательность, связи, кто, когда, зачем (бизнес), к какой контрольной точке. Строки с пометкой ПРИМЕР замените своими.</t>
+          <t>доска остаётся отчётной доской. Этот файл — последовательность, связи, кто, когда, зачем (бизнес), к какой контрольной точке. Строки с пометкой ПРИМЕР замените своими.</t>
         </is>
       </c>
     </row>
@@ -986,7 +1021,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Картина недели: сколько задач по стримам, что блокирует ОЭ, что ★</t>
+          <t>Картина недели: сколько задач по стримам, что блокирует цель, что ★</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -1020,7 +1055,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Вехи и КТ проекта, в т.ч. выход в опытную эксплуатацию</t>
+          <t>Вехи и КТ проекта, в т.ч. выход в цель проекта</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -1066,7 +1101,7 @@
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Ресурсы</t>
+          <t>Подстрим 5.2</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -1128,7 +1163,7 @@
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>4. Общепроектные (финансы, обучение, закупки…) — отдельные строки только если есть ваш срок или вас спрашивают на дэйли.</t>
+          <t>4. Стрим 5 (финансы, обучение, закупки…) — отдельные строки только если есть ваш срок или вас спрашивают на ежедневный статус.</t>
         </is>
       </c>
     </row>
@@ -1142,14 +1177,14 @@
     <row r="19" ht="22" customHeight="1">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>6. Master-артефакты (концепт, схемы, сайзинг) указывайте в «Источник» как путь на общий диск, не копируйте файл сюда.</t>
+          <t>6. Master-артефакты (документ этапа, схемы, расчёт параметров) указывайте в «Источник» как путь на общий диск, не копируйте файл сюда.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="22" customHeight="1">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>7. После 01.09 верните чужие стримы второму ТРП: статус «Передано», в «Ответственный» — его имя.</t>
+          <t>7. После 01.09 верните чужие стримы второму роль ведения: статус «Передано», в «Ответственный» — его имя.</t>
         </is>
       </c>
     </row>
@@ -1163,7 +1198,7 @@
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>Архитектура</t>
+          <t>Стрим 1</t>
         </is>
       </c>
       <c r="B23" s="9" t="n"/>
@@ -1171,7 +1206,7 @@
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
         <is>
-          <t>Инфраструктура</t>
+          <t>Стрим 2</t>
         </is>
       </c>
       <c r="B24" s="9" t="n"/>
@@ -1179,7 +1214,7 @@
     <row r="25">
       <c r="A25" s="11" t="inlineStr">
         <is>
-          <t>ИБ</t>
+          <t>Стрим 3</t>
         </is>
       </c>
       <c r="B25" s="9" t="n"/>
@@ -1187,7 +1222,7 @@
     <row r="26">
       <c r="A26" s="12" t="inlineStr">
         <is>
-          <t>Качество данных</t>
+          <t>Стрим 4</t>
         </is>
       </c>
       <c r="B26" s="9" t="n"/>
@@ -1195,7 +1230,7 @@
     <row r="27">
       <c r="A27" s="13" t="inlineStr">
         <is>
-          <t>Общепроектные</t>
+          <t>Стрим 5</t>
         </is>
       </c>
       <c r="B27" s="9" t="n"/>
@@ -1203,7 +1238,7 @@
     <row r="28">
       <c r="A28" s="14" t="inlineStr">
         <is>
-          <t>★ фокус недели / КТ ОЭ</t>
+          <t>★ фокус недели / КТ цели</t>
         </is>
       </c>
       <c r="B28" s="9" t="n"/>
@@ -1211,16 +1246,16 @@
     <row r="30" ht="36" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Как читать календарь справа на листе «План_работ»: точка в неделе = задача идёт в эти даты. Жёлтая заливка недели = пересечение с контрольной точкой ОЭ (см. лист КТ).</t>
+          <t>Как читать календарь справа на листе «План_работ»: точка в неделе = задача идёт в эти даты. Жёлтая заливка недели = пересечение с контрольной точкой цель (см. лист КТ).</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A26:B26"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A16:F16"/>
     <mergeCell ref="A24:B24"/>
-    <mergeCell ref="A26:B26"/>
     <mergeCell ref="A30:F30"/>
     <mergeCell ref="A13:F13"/>
     <mergeCell ref="A14:F14"/>
@@ -1263,14 +1298,14 @@
     <row r="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>Сводка на неделю — открывать вместо «просмотреть всю доску»</t>
+          <t>Сводка на неделю — открывать вместо полной доски задач</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="16" t="inlineStr">
         <is>
-          <t>Цифры считаются с листа «План_работ». Пустые строки не мешают. После замены примеров проверьте ★ (должно быть 3).</t>
+          <t>Цифры считаются с листа «План_работ». Пустые строки не мешают. ★ — не больше трёх.</t>
         </is>
       </c>
     </row>
@@ -1304,7 +1339,7 @@
       </c>
       <c r="E5" s="17" t="inlineStr">
         <is>
-          <t>Блокируют ОЭ</t>
+          <t>Блокируют цель</t>
         </is>
       </c>
       <c r="F5" s="17" t="inlineStr">
@@ -1316,7 +1351,7 @@
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="18" t="inlineStr">
         <is>
-          <t>Архитектура</t>
+          <t>Стрим 1</t>
         </is>
       </c>
       <c r="B6" s="19">
@@ -1343,7 +1378,7 @@
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="20" t="inlineStr">
         <is>
-          <t>Инфраструктура</t>
+          <t>Стрим 2</t>
         </is>
       </c>
       <c r="B7" s="19">
@@ -1370,7 +1405,7 @@
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>ИБ</t>
+          <t>Стрим 3</t>
         </is>
       </c>
       <c r="B8" s="19">
@@ -1397,7 +1432,7 @@
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="22" t="inlineStr">
         <is>
-          <t>Качество данных</t>
+          <t>Стрим 4</t>
         </is>
       </c>
       <c r="B9" s="19">
@@ -1424,7 +1459,7 @@
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="23" t="inlineStr">
         <is>
-          <t>Общепроектные</t>
+          <t>Стрим 5</t>
         </is>
       </c>
       <c r="B10" s="19">
@@ -1507,7 +1542,7 @@
     <row r="16" ht="22" customHeight="1">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>Блокируют опытную эксплуатацию</t>
+          <t>Блокируют цель проекта</t>
         </is>
       </c>
       <c r="E16" s="25">
@@ -1532,7 +1567,7 @@
           <t>Ближайшая КТ (дата)</t>
         </is>
       </c>
-      <c r="E18" s="26">
+      <c r="E18" s="71">
         <f>MIN(Контрольные_точки!D5:D15)</f>
         <v/>
       </c>
@@ -1580,7 +1615,7 @@
         <f>Контрольные_точки!C5</f>
         <v/>
       </c>
-      <c r="C22" s="28">
+      <c r="C22" s="72">
         <f>Контрольные_точки!D5</f>
         <v/>
       </c>
@@ -1602,7 +1637,7 @@
         <f>Контрольные_точки!C6</f>
         <v/>
       </c>
-      <c r="C23" s="28">
+      <c r="C23" s="72">
         <f>Контрольные_точки!D6</f>
         <v/>
       </c>
@@ -1624,7 +1659,7 @@
         <f>Контрольные_точки!C7</f>
         <v/>
       </c>
-      <c r="C24" s="28">
+      <c r="C24" s="72">
         <f>Контрольные_точки!D7</f>
         <v/>
       </c>
@@ -1646,7 +1681,7 @@
         <f>Контрольные_точки!C8</f>
         <v/>
       </c>
-      <c r="C25" s="28">
+      <c r="C25" s="72">
         <f>Контрольные_точки!D8</f>
         <v/>
       </c>
@@ -1668,7 +1703,7 @@
         <f>Контрольные_точки!C9</f>
         <v/>
       </c>
-      <c r="C26" s="28">
+      <c r="C26" s="72">
         <f>Контрольные_точки!D9</f>
         <v/>
       </c>
@@ -1705,9 +1740,9 @@
       <c r="A32" s="30" t="inlineStr">
         <is>
           <t>Статус [дата]
-• Архитектура: … / следующий шаг: …
-• ИБ: … / жду: …
-• Инфра: …
+• Стрим 1: … / следующий шаг: …
+• Стрим 3: … / жду: …
+• Стрим 2: …
 • На неделе закрываю: (три ★)
 • Блокер: нет / есть: …</t>
         </is>
@@ -1803,14 +1838,14 @@
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>ПРИМЕР заполнения под вашу цепочку (концепт → сети → сайзинг → ОЭ). Замените ФИО, даты и «следующий шаг». Колонка ★ — не больше трёх. Календарь справа пересчитывается от дат начала/окончания.</t>
+          <t>Обезличенный ПРИМЕР. Замените участников, даты и «следующий шаг». Колонка ★ — не больше трёх. Календарь справа от дат начала/окончания.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="8" customHeight="1">
       <c r="V3" s="16" t="inlineStr">
         <is>
-          <t>Календарь: ● = задача идёт в эту неделю. Жёлтая шапка = неделя старта ОЭ (KT-OE).</t>
+          <t>Календарь: ● = задача идёт в эту неделю. Жёлтая шапка = неделя цели (KT-05).</t>
         </is>
       </c>
     </row>
@@ -1902,7 +1937,7 @@
       </c>
       <c r="R4" s="17" t="inlineStr">
         <is>
-          <t>Блокирует ОЭ</t>
+          <t>Блокирует цель</t>
         </is>
       </c>
       <c r="S4" s="17" t="inlineStr">
@@ -1920,56 +1955,56 @@
           <t>Комментарий</t>
         </is>
       </c>
-      <c r="V4" s="31" t="n">
+      <c r="V4" s="73" t="n">
         <v>46258</v>
       </c>
-      <c r="W4" s="31" t="n">
+      <c r="W4" s="73" t="n">
         <v>46265</v>
       </c>
-      <c r="X4" s="31" t="n">
+      <c r="X4" s="73" t="n">
         <v>46272</v>
       </c>
-      <c r="Y4" s="31" t="n">
+      <c r="Y4" s="73" t="n">
         <v>46279</v>
       </c>
-      <c r="Z4" s="31" t="n">
+      <c r="Z4" s="73" t="n">
         <v>46286</v>
       </c>
-      <c r="AA4" s="31" t="n">
+      <c r="AA4" s="73" t="n">
         <v>46293</v>
       </c>
-      <c r="AB4" s="31" t="n">
+      <c r="AB4" s="73" t="n">
         <v>46300</v>
       </c>
-      <c r="AC4" s="31" t="n">
+      <c r="AC4" s="73" t="n">
         <v>46307</v>
       </c>
-      <c r="AD4" s="32" t="n">
+      <c r="AD4" s="74" t="n">
         <v>46314</v>
       </c>
-      <c r="AE4" s="33" t="n">
+      <c r="AE4" s="75" t="n">
         <v>46321</v>
       </c>
-      <c r="AF4" s="31" t="n">
+      <c r="AF4" s="73" t="n">
         <v>46328</v>
       </c>
-      <c r="AG4" s="31" t="n">
+      <c r="AG4" s="73" t="n">
         <v>46335</v>
       </c>
-      <c r="AH4" s="31" t="n">
+      <c r="AH4" s="73" t="n">
         <v>46342</v>
       </c>
     </row>
     <row r="5" ht="46" customHeight="1">
       <c r="A5" s="34" t="inlineStr">
         <is>
-          <t>A-01</t>
-        </is>
-      </c>
-      <c r="B5" s="34" t="inlineStr"/>
+          <t>S1-01</t>
+        </is>
+      </c>
+      <c r="B5" s="34" t="n"/>
       <c r="C5" s="18" t="inlineStr">
         <is>
-          <t>Архитектура</t>
+          <t>Стрим 1</t>
         </is>
       </c>
       <c r="D5" s="18" t="inlineStr">
@@ -1979,7 +2014,7 @@
       </c>
       <c r="E5" s="18" t="inlineStr">
         <is>
-          <t>Концептуальный дизайн: довести документ до согласованной версии</t>
+          <t>Задача 1.1: подготовить документ этапа</t>
         </is>
       </c>
       <c r="F5" s="34" t="inlineStr">
@@ -1992,10 +2027,10 @@
           <t>KT-02</t>
         </is>
       </c>
-      <c r="H5" s="35" t="n">
+      <c r="H5" s="76" t="n">
         <v>46258</v>
       </c>
-      <c r="I5" s="35" t="n">
+      <c r="I5" s="76" t="n">
         <v>46277</v>
       </c>
       <c r="J5" s="36">
@@ -2004,12 +2039,12 @@
       </c>
       <c r="K5" s="18" t="inlineStr">
         <is>
-          <t>Я</t>
+          <t>Участник A</t>
         </is>
       </c>
       <c r="L5" s="18" t="inlineStr">
         <is>
-          <t>Архитектор / ТРП</t>
+          <t>Роль A</t>
         </is>
       </c>
       <c r="M5" s="37" t="n">
@@ -2032,17 +2067,17 @@
       </c>
       <c r="S5" s="18" t="inlineStr">
         <is>
-          <t>Собрать открытые замечания ИБ и инфры в один список</t>
+          <t>Собрать открытые замечания в один список</t>
         </is>
       </c>
       <c r="T5" s="18" t="inlineStr">
         <is>
-          <t>Общий диск \arch\concept.docx; протоколы в ИИ</t>
+          <t>Источник: общий диск / протоколы</t>
         </is>
       </c>
       <c r="U5" s="18" t="inlineStr">
         <is>
-          <t>Вход для схем и сайзинга</t>
+          <t>Вход для следующих задач стрима</t>
         </is>
       </c>
       <c r="V5" s="38">
@@ -2101,13 +2136,13 @@
     <row r="6" ht="46" customHeight="1">
       <c r="A6" s="34" t="inlineStr">
         <is>
-          <t>A-02</t>
-        </is>
-      </c>
-      <c r="B6" s="34" t="inlineStr"/>
+          <t>S1-02</t>
+        </is>
+      </c>
+      <c r="B6" s="34" t="n"/>
       <c r="C6" s="18" t="inlineStr">
         <is>
-          <t>Архитектура</t>
+          <t>Стрим 1</t>
         </is>
       </c>
       <c r="D6" s="18" t="inlineStr">
@@ -2117,7 +2152,7 @@
       </c>
       <c r="E6" s="18" t="inlineStr">
         <is>
-          <t>Сетевые схемы по концепту</t>
+          <t>Задача 1.2: подготовить схемы по документу</t>
         </is>
       </c>
       <c r="F6" s="34" t="inlineStr">
@@ -2130,10 +2165,10 @@
           <t>KT-03</t>
         </is>
       </c>
-      <c r="H6" s="35" t="n">
+      <c r="H6" s="76" t="n">
         <v>46273</v>
       </c>
-      <c r="I6" s="35" t="n">
+      <c r="I6" s="76" t="n">
         <v>46284</v>
       </c>
       <c r="J6" s="36">
@@ -2142,12 +2177,12 @@
       </c>
       <c r="K6" s="18" t="inlineStr">
         <is>
-          <t>Я</t>
+          <t>Участник A</t>
         </is>
       </c>
       <c r="L6" s="18" t="inlineStr">
         <is>
-          <t>Сетевой архитектор (ФИО)</t>
+          <t>Роль B</t>
         </is>
       </c>
       <c r="M6" s="37" t="n">
@@ -2155,7 +2190,7 @@
       </c>
       <c r="N6" s="18" t="inlineStr">
         <is>
-          <t>A-01</t>
+          <t>S1-01</t>
         </is>
       </c>
       <c r="O6" s="18" t="inlineStr">
@@ -2178,17 +2213,17 @@
       </c>
       <c r="S6" s="18" t="inlineStr">
         <is>
-          <t>Начать после стабилизации разделов концепта по сегментации</t>
+          <t>Начать после стабилизации ключевых разделов документа</t>
         </is>
       </c>
       <c r="T6" s="18" t="inlineStr">
         <is>
-          <t>Общий диск \arch\net\</t>
+          <t>Источник: папка схем</t>
         </is>
       </c>
       <c r="U6" s="18" t="inlineStr">
         <is>
-          <t>Можно стартовать с лагом −4 дня, если концепт почти готов</t>
+          <t>Можно стартовать с лагом, если документ почти готов</t>
         </is>
       </c>
       <c r="V6" s="38">
@@ -2247,7 +2282,7 @@
     <row r="7" ht="46" customHeight="1">
       <c r="A7" s="34" t="inlineStr">
         <is>
-          <t>A-03</t>
+          <t>S1-03</t>
         </is>
       </c>
       <c r="B7" s="39" t="inlineStr">
@@ -2257,7 +2292,7 @@
       </c>
       <c r="C7" s="18" t="inlineStr">
         <is>
-          <t>Архитектура</t>
+          <t>Стрим 1</t>
         </is>
       </c>
       <c r="D7" s="18" t="inlineStr">
@@ -2267,7 +2302,7 @@
       </c>
       <c r="E7" s="18" t="inlineStr">
         <is>
-          <t>Сайзинг контура</t>
+          <t>Задача 1.3: рассчитать параметры контура</t>
         </is>
       </c>
       <c r="F7" s="34" t="inlineStr">
@@ -2280,10 +2315,10 @@
           <t>KT-03</t>
         </is>
       </c>
-      <c r="H7" s="35" t="n">
+      <c r="H7" s="76" t="n">
         <v>46280</v>
       </c>
-      <c r="I7" s="35" t="n">
+      <c r="I7" s="76" t="n">
         <v>46291</v>
       </c>
       <c r="J7" s="36">
@@ -2292,12 +2327,12 @@
       </c>
       <c r="K7" s="18" t="inlineStr">
         <is>
-          <t>Я</t>
+          <t>Участник A</t>
         </is>
       </c>
       <c r="L7" s="18" t="inlineStr">
         <is>
-          <t>Архитектор + инфра</t>
+          <t>Роль A + Роль C</t>
         </is>
       </c>
       <c r="M7" s="37" t="n">
@@ -2305,7 +2340,7 @@
       </c>
       <c r="N7" s="18" t="inlineStr">
         <is>
-          <t>A-02</t>
+          <t>S1-02</t>
         </is>
       </c>
       <c r="O7" s="18" t="inlineStr">
@@ -2328,17 +2363,17 @@
       </c>
       <c r="S7" s="18" t="inlineStr">
         <is>
-          <t>Набросать структуру таблицы CPU/RAM/диск по зонам</t>
+          <t>Набросать структуру таблицы параметров по зонам</t>
         </is>
       </c>
       <c r="T7" s="18" t="inlineStr">
         <is>
-          <t>Общий диск \arch\sizing.xlsx</t>
+          <t>Источник: таблица параметров</t>
         </is>
       </c>
       <c r="U7" s="18" t="inlineStr">
         <is>
-          <t>Типичный фокус недели, когда схемы уже есть</t>
+          <t>Типичный фокус недели</t>
         </is>
       </c>
       <c r="V7" s="38">
@@ -2397,13 +2432,13 @@
     <row r="8" ht="46" customHeight="1">
       <c r="A8" s="34" t="inlineStr">
         <is>
-          <t>A-04</t>
-        </is>
-      </c>
-      <c r="B8" s="34" t="inlineStr"/>
+          <t>S1-04</t>
+        </is>
+      </c>
+      <c r="B8" s="34" t="n"/>
       <c r="C8" s="18" t="inlineStr">
         <is>
-          <t>Архитектура</t>
+          <t>Стрим 1</t>
         </is>
       </c>
       <c r="D8" s="18" t="inlineStr">
@@ -2413,7 +2448,7 @@
       </c>
       <c r="E8" s="18" t="inlineStr">
         <is>
-          <t>Пакет артефактов архитектуры в ОЭ</t>
+          <t>Задача 1.4: собрать пакет артефактов к цели</t>
         </is>
       </c>
       <c r="F8" s="34" t="inlineStr">
@@ -2423,13 +2458,13 @@
       </c>
       <c r="G8" s="34" t="inlineStr">
         <is>
-          <t>KT-OE</t>
-        </is>
-      </c>
-      <c r="H8" s="35" t="n">
+          <t>KT-05</t>
+        </is>
+      </c>
+      <c r="H8" s="76" t="n">
         <v>46301</v>
       </c>
-      <c r="I8" s="35" t="n">
+      <c r="I8" s="76" t="n">
         <v>46312</v>
       </c>
       <c r="J8" s="36">
@@ -2438,12 +2473,12 @@
       </c>
       <c r="K8" s="18" t="inlineStr">
         <is>
-          <t>Я</t>
+          <t>Участник A</t>
         </is>
       </c>
       <c r="L8" s="18" t="inlineStr">
         <is>
-          <t>ТРП</t>
+          <t>Роль A</t>
         </is>
       </c>
       <c r="M8" s="37" t="n">
@@ -2451,7 +2486,7 @@
       </c>
       <c r="N8" s="18" t="inlineStr">
         <is>
-          <t>A-03,I-03,IB-03</t>
+          <t>S1-03,S2-03,S3-03</t>
         </is>
       </c>
       <c r="O8" s="18" t="inlineStr">
@@ -2474,17 +2509,17 @@
       </c>
       <c r="S8" s="18" t="inlineStr">
         <is>
-          <t>Собрать чеклист: концепт, схемы, сайзинг, ссылки</t>
+          <t>Собрать чеклист артефактов и ссылок</t>
         </is>
       </c>
       <c r="T8" s="18" t="inlineStr">
         <is>
-          <t>КТ ОЭ в Confluence + диск</t>
+          <t>Источник: КТ цели + диск</t>
         </is>
       </c>
       <c r="U8" s="18" t="inlineStr">
         <is>
-          <t>Сходится с инфрой и ИБ</t>
+          <t>Сходится со стримами 2 и 3</t>
         </is>
       </c>
       <c r="V8" s="38">
@@ -2543,13 +2578,13 @@
     <row r="9" ht="46" customHeight="1">
       <c r="A9" s="40" t="inlineStr">
         <is>
-          <t>I-01</t>
-        </is>
-      </c>
-      <c r="B9" s="40" t="inlineStr"/>
+          <t>S2-01</t>
+        </is>
+      </c>
+      <c r="B9" s="40" t="n"/>
       <c r="C9" s="20" t="inlineStr">
         <is>
-          <t>Инфраструктура</t>
+          <t>Стрим 2</t>
         </is>
       </c>
       <c r="D9" s="20" t="inlineStr">
@@ -2559,7 +2594,7 @@
       </c>
       <c r="E9" s="20" t="inlineStr">
         <is>
-          <t>Требования к контуру / стенду ОЭ</t>
+          <t>Задача 2.1: зафиксировать требования к среде</t>
         </is>
       </c>
       <c r="F9" s="40" t="inlineStr">
@@ -2572,10 +2607,10 @@
           <t>KT-03</t>
         </is>
       </c>
-      <c r="H9" s="41" t="n">
+      <c r="H9" s="77" t="n">
         <v>46265</v>
       </c>
-      <c r="I9" s="41" t="n">
+      <c r="I9" s="77" t="n">
         <v>46277</v>
       </c>
       <c r="J9" s="42">
@@ -2584,12 +2619,12 @@
       </c>
       <c r="K9" s="20" t="inlineStr">
         <is>
-          <t>Инфра (ФИО)</t>
+          <t>Участник C</t>
         </is>
       </c>
       <c r="L9" s="20" t="inlineStr">
         <is>
-          <t>Инженер инфры</t>
+          <t>Роль C</t>
         </is>
       </c>
       <c r="M9" s="43" t="n">
@@ -2597,7 +2632,7 @@
       </c>
       <c r="N9" s="20" t="inlineStr">
         <is>
-          <t>A-01</t>
+          <t>S1-01</t>
         </is>
       </c>
       <c r="O9" s="20" t="inlineStr">
@@ -2620,17 +2655,17 @@
       </c>
       <c r="S9" s="20" t="inlineStr">
         <is>
-          <t>Запросить у инфры список открытых вопросов к концепту</t>
+          <t>Запросить список открытых вопросов к документу</t>
         </is>
       </c>
       <c r="T9" s="20" t="inlineStr">
         <is>
-          <t>Встреча арх+инфра, протокол</t>
+          <t>Источник: протокол встречи</t>
         </is>
       </c>
       <c r="U9" s="20" t="inlineStr">
         <is>
-          <t>Параллельно концепту, не ждать финала</t>
+          <t>Параллельно документу стрима 1</t>
         </is>
       </c>
       <c r="V9" s="38">
@@ -2689,13 +2724,13 @@
     <row r="10" ht="46" customHeight="1">
       <c r="A10" s="40" t="inlineStr">
         <is>
-          <t>I-02</t>
-        </is>
-      </c>
-      <c r="B10" s="40" t="inlineStr"/>
+          <t>S2-02</t>
+        </is>
+      </c>
+      <c r="B10" s="40" t="n"/>
       <c r="C10" s="20" t="inlineStr">
         <is>
-          <t>Инфраструктура</t>
+          <t>Стрим 2</t>
         </is>
       </c>
       <c r="D10" s="20" t="inlineStr">
@@ -2705,7 +2740,7 @@
       </c>
       <c r="E10" s="20" t="inlineStr">
         <is>
-          <t>Контур / стенд: развёртывание</t>
+          <t>Задача 2.2: подготовить / развернуть среду</t>
         </is>
       </c>
       <c r="F10" s="40" t="inlineStr">
@@ -2715,13 +2750,13 @@
       </c>
       <c r="G10" s="40" t="inlineStr">
         <is>
-          <t>KT-OE</t>
-        </is>
-      </c>
-      <c r="H10" s="41" t="n">
+          <t>KT-05</t>
+        </is>
+      </c>
+      <c r="H10" s="77" t="n">
         <v>46279</v>
       </c>
-      <c r="I10" s="41" t="n">
+      <c r="I10" s="77" t="n">
         <v>46304</v>
       </c>
       <c r="J10" s="42">
@@ -2730,12 +2765,12 @@
       </c>
       <c r="K10" s="20" t="inlineStr">
         <is>
-          <t>Инфра (ФИО)</t>
+          <t>Участник C</t>
         </is>
       </c>
       <c r="L10" s="20" t="inlineStr">
         <is>
-          <t>Стенд / контур</t>
+          <t>Среда / стенд</t>
         </is>
       </c>
       <c r="M10" s="43" t="n">
@@ -2743,7 +2778,7 @@
       </c>
       <c r="N10" s="20" t="inlineStr">
         <is>
-          <t>I-01,A-03</t>
+          <t>S2-01,S1-03</t>
         </is>
       </c>
       <c r="O10" s="20" t="inlineStr">
@@ -2766,17 +2801,17 @@
       </c>
       <c r="S10" s="20" t="inlineStr">
         <is>
-          <t>Уточнить дату появления стенда письмом</t>
+          <t>Уточнить дату готовности среды письмом</t>
         </is>
       </c>
       <c r="T10" s="20" t="inlineStr">
         <is>
-          <t>Чат инфры, письмо</t>
+          <t>Источник: чат / письмо</t>
         </is>
       </c>
       <c r="U10" s="20" t="inlineStr">
         <is>
-          <t>Сайзинг должен подтвердить мощность</t>
+          <t>Параметры стрима 1 должны подтвердить объём</t>
         </is>
       </c>
       <c r="V10" s="38">
@@ -2835,7 +2870,7 @@
     <row r="11" ht="46" customHeight="1">
       <c r="A11" s="40" t="inlineStr">
         <is>
-          <t>I-03</t>
+          <t>S2-03</t>
         </is>
       </c>
       <c r="B11" s="39" t="inlineStr">
@@ -2845,7 +2880,7 @@
       </c>
       <c r="C11" s="20" t="inlineStr">
         <is>
-          <t>Инфраструктура</t>
+          <t>Стрим 2</t>
         </is>
       </c>
       <c r="D11" s="20" t="inlineStr">
@@ -2855,7 +2890,7 @@
       </c>
       <c r="E11" s="20" t="inlineStr">
         <is>
-          <t>Готовность инфраструктуры к ОЭ</t>
+          <t>Задача 2.3: подтвердить готовность среды к цели</t>
         </is>
       </c>
       <c r="F11" s="40" t="inlineStr">
@@ -2865,13 +2900,13 @@
       </c>
       <c r="G11" s="40" t="inlineStr">
         <is>
-          <t>KT-OE</t>
-        </is>
-      </c>
-      <c r="H11" s="41" t="n">
+          <t>KT-05</t>
+        </is>
+      </c>
+      <c r="H11" s="77" t="n">
         <v>46301</v>
       </c>
-      <c r="I11" s="41" t="n">
+      <c r="I11" s="77" t="n">
         <v>46312</v>
       </c>
       <c r="J11" s="42">
@@ -2880,12 +2915,12 @@
       </c>
       <c r="K11" s="20" t="inlineStr">
         <is>
-          <t>Инфра (ФИО)</t>
+          <t>Участник C</t>
         </is>
       </c>
       <c r="L11" s="20" t="inlineStr">
         <is>
-          <t>Инженер инфры + ТРП</t>
+          <t>Роль C + Роль A</t>
         </is>
       </c>
       <c r="M11" s="43" t="n">
@@ -2893,7 +2928,7 @@
       </c>
       <c r="N11" s="20" t="inlineStr">
         <is>
-          <t>I-02</t>
+          <t>S2-02</t>
         </is>
       </c>
       <c r="O11" s="20" t="inlineStr">
@@ -2916,12 +2951,12 @@
       </c>
       <c r="S11" s="20" t="inlineStr">
         <is>
-          <t>Согласовать чеклист готовности (доступ, мониторинг, бэкап)</t>
+          <t>Согласовать чеклист готовности</t>
         </is>
       </c>
       <c r="T11" s="20" t="inlineStr">
         <is>
-          <t>Регламент ОЭ</t>
+          <t>Источник: регламент цели</t>
         </is>
       </c>
       <c r="U11" s="20" t="inlineStr"/>
@@ -2981,13 +3016,13 @@
     <row r="12" ht="46" customHeight="1">
       <c r="A12" s="44" t="inlineStr">
         <is>
-          <t>IB-01</t>
-        </is>
-      </c>
-      <c r="B12" s="44" t="inlineStr"/>
+          <t>S3-01</t>
+        </is>
+      </c>
+      <c r="B12" s="44" t="n"/>
       <c r="C12" s="21" t="inlineStr">
         <is>
-          <t>ИБ</t>
+          <t>Стрим 3</t>
         </is>
       </c>
       <c r="D12" s="21" t="inlineStr">
@@ -2997,7 +3032,7 @@
       </c>
       <c r="E12" s="21" t="inlineStr">
         <is>
-          <t>Реестр задач ИБ к ОЭ</t>
+          <t>Задача 3.1: собрать реестр задач стрима 3</t>
         </is>
       </c>
       <c r="F12" s="44" t="inlineStr">
@@ -3010,10 +3045,10 @@
           <t>KT-04</t>
         </is>
       </c>
-      <c r="H12" s="45" t="n">
+      <c r="H12" s="78" t="n">
         <v>46258</v>
       </c>
-      <c r="I12" s="45" t="n">
+      <c r="I12" s="78" t="n">
         <v>46270</v>
       </c>
       <c r="J12" s="46">
@@ -3022,12 +3057,12 @@
       </c>
       <c r="K12" s="21" t="inlineStr">
         <is>
-          <t>Я</t>
+          <t>Участник A</t>
         </is>
       </c>
       <c r="L12" s="21" t="inlineStr">
         <is>
-          <t>ТРП + ИБ</t>
+          <t>Роль A + Роль D</t>
         </is>
       </c>
       <c r="M12" s="47" t="n">
@@ -3050,17 +3085,17 @@
       </c>
       <c r="S12" s="21" t="inlineStr">
         <is>
-          <t>Сверить доску ИБ со статус-встречей, выкинуть не-ОЭ</t>
+          <t>Сверить доску со статусной встречей, убрать лишнее</t>
         </is>
       </c>
       <c r="T12" s="21" t="inlineStr">
         <is>
-          <t>Доска Confluence ИБ; протоколы статусов</t>
+          <t>Источник: доска / протоколы</t>
         </is>
       </c>
       <c r="U12" s="21" t="inlineStr">
         <is>
-          <t>Покрытие до 01.09 — не раздувать</t>
+          <t>Не раздувать объём</t>
         </is>
       </c>
       <c r="V12" s="38">
@@ -3119,7 +3154,7 @@
     <row r="13" ht="46" customHeight="1">
       <c r="A13" s="44" t="inlineStr">
         <is>
-          <t>IB-02</t>
+          <t>S3-02</t>
         </is>
       </c>
       <c r="B13" s="39" t="inlineStr">
@@ -3129,7 +3164,7 @@
       </c>
       <c r="C13" s="21" t="inlineStr">
         <is>
-          <t>ИБ</t>
+          <t>Стрим 3</t>
         </is>
       </c>
       <c r="D13" s="21" t="inlineStr">
@@ -3139,7 +3174,7 @@
       </c>
       <c r="E13" s="21" t="inlineStr">
         <is>
-          <t>Закрытие замечаний ИБ (концепт / схемы / контур)</t>
+          <t>Задача 3.2: закрыть замечания по артефактам</t>
         </is>
       </c>
       <c r="F13" s="44" t="inlineStr">
@@ -3152,10 +3187,10 @@
           <t>KT-04</t>
         </is>
       </c>
-      <c r="H13" s="45" t="n">
+      <c r="H13" s="78" t="n">
         <v>46273</v>
       </c>
-      <c r="I13" s="45" t="n">
+      <c r="I13" s="78" t="n">
         <v>46298</v>
       </c>
       <c r="J13" s="46">
@@ -3164,12 +3199,12 @@
       </c>
       <c r="K13" s="21" t="inlineStr">
         <is>
-          <t>Я</t>
+          <t>Участник A</t>
         </is>
       </c>
       <c r="L13" s="21" t="inlineStr">
         <is>
-          <t>ИБ (ФИО) + архитектор</t>
+          <t>Роль D + Роль A</t>
         </is>
       </c>
       <c r="M13" s="47" t="n">
@@ -3177,7 +3212,7 @@
       </c>
       <c r="N13" s="21" t="inlineStr">
         <is>
-          <t>IB-01,A-01,A-02</t>
+          <t>S3-01,S1-01,S1-02</t>
         </is>
       </c>
       <c r="O13" s="21" t="inlineStr">
@@ -3200,17 +3235,17 @@
       </c>
       <c r="S13" s="21" t="inlineStr">
         <is>
-          <t>Ответить на 3 открытых пункта из последнего протокола статусов</t>
+          <t>Ответить на открытые пункты из последнего протокола</t>
         </is>
       </c>
       <c r="T13" s="21" t="inlineStr">
         <is>
-          <t>Протокол статусов ИБ; ИИ: «замечания ИБ ОЭ»</t>
+          <t>Источник: протокол статусов</t>
         </is>
       </c>
       <c r="U13" s="21" t="inlineStr">
         <is>
-          <t>Статус «Жду» — кто именно, написать в комментарии</t>
+          <t>В статусе «Жду» указать кого</t>
         </is>
       </c>
       <c r="V13" s="38">
@@ -3269,13 +3304,13 @@
     <row r="14" ht="46" customHeight="1">
       <c r="A14" s="44" t="inlineStr">
         <is>
-          <t>IB-03</t>
-        </is>
-      </c>
-      <c r="B14" s="44" t="inlineStr"/>
+          <t>S3-03</t>
+        </is>
+      </c>
+      <c r="B14" s="44" t="n"/>
       <c r="C14" s="21" t="inlineStr">
         <is>
-          <t>ИБ</t>
+          <t>Стрим 3</t>
         </is>
       </c>
       <c r="D14" s="21" t="inlineStr">
@@ -3285,7 +3320,7 @@
       </c>
       <c r="E14" s="21" t="inlineStr">
         <is>
-          <t>Допуск ИБ в опытную эксплуатацию</t>
+          <t>Задача 3.3: оформить допуск к цели</t>
         </is>
       </c>
       <c r="F14" s="44" t="inlineStr">
@@ -3298,10 +3333,10 @@
           <t>KT-04</t>
         </is>
       </c>
-      <c r="H14" s="45" t="n">
+      <c r="H14" s="78" t="n">
         <v>46301</v>
       </c>
-      <c r="I14" s="45" t="n">
+      <c r="I14" s="78" t="n">
         <v>46305</v>
       </c>
       <c r="J14" s="46">
@@ -3310,12 +3345,12 @@
       </c>
       <c r="K14" s="21" t="inlineStr">
         <is>
-          <t>ИБ (ФИО)</t>
+          <t>Участник D</t>
         </is>
       </c>
       <c r="L14" s="21" t="inlineStr">
         <is>
-          <t>ИБ</t>
+          <t>Роль D</t>
         </is>
       </c>
       <c r="M14" s="47" t="n">
@@ -3323,7 +3358,7 @@
       </c>
       <c r="N14" s="21" t="inlineStr">
         <is>
-          <t>IB-02,I-02</t>
+          <t>S3-02,S2-02</t>
         </is>
       </c>
       <c r="O14" s="21" t="inlineStr">
@@ -3351,12 +3386,12 @@
       </c>
       <c r="T14" s="21" t="inlineStr">
         <is>
-          <t>Регламент ИБ / папка ОЭ</t>
+          <t>Источник: регламент / папка цели</t>
         </is>
       </c>
       <c r="U14" s="21" t="inlineStr">
         <is>
-          <t>Блокер старта ОЭ</t>
+          <t>Блокер старта цели</t>
         </is>
       </c>
       <c r="V14" s="38">
@@ -3415,13 +3450,13 @@
     <row r="15" ht="46" customHeight="1">
       <c r="A15" s="48" t="inlineStr">
         <is>
-          <t>DQ-01</t>
-        </is>
-      </c>
-      <c r="B15" s="48" t="inlineStr"/>
+          <t>S4-01</t>
+        </is>
+      </c>
+      <c r="B15" s="48" t="n"/>
       <c r="C15" s="22" t="inlineStr">
         <is>
-          <t>Качество данных</t>
+          <t>Стрим 4</t>
         </is>
       </c>
       <c r="D15" s="22" t="inlineStr">
@@ -3431,7 +3466,7 @@
       </c>
       <c r="E15" s="22" t="inlineStr">
         <is>
-          <t>Проверки качества к ОЭ: нужно ли нам это до старта</t>
+          <t>Задача 4.1: понять, нужны ли проверки до цели</t>
         </is>
       </c>
       <c r="F15" s="48" t="inlineStr">
@@ -3441,13 +3476,13 @@
       </c>
       <c r="G15" s="48" t="inlineStr">
         <is>
-          <t>KT-OE</t>
-        </is>
-      </c>
-      <c r="H15" s="49" t="n">
+          <t>KT-05</t>
+        </is>
+      </c>
+      <c r="H15" s="79" t="n">
         <v>46280</v>
       </c>
-      <c r="I15" s="49" t="n">
+      <c r="I15" s="79" t="n">
         <v>46284</v>
       </c>
       <c r="J15" s="50">
@@ -3456,12 +3491,12 @@
       </c>
       <c r="K15" s="22" t="inlineStr">
         <is>
-          <t>Я / DQ (ФИО)</t>
+          <t>Участник A / Участник E</t>
         </is>
       </c>
       <c r="L15" s="22" t="inlineStr">
         <is>
-          <t>Аналитик данных</t>
+          <t>Роль E</t>
         </is>
       </c>
       <c r="M15" s="51" t="n">
@@ -3484,12 +3519,12 @@
       </c>
       <c r="S15" s="22" t="inlineStr">
         <is>
-          <t>Выяснить у владельца DQ, блокирует ли ОЭ; если нет — «Отложено»</t>
+          <t>Выяснить у владельца, блокирует ли цель; если нет — «Отложено»</t>
         </is>
       </c>
       <c r="T15" s="22" t="inlineStr">
         <is>
-          <t>Confluence DQ</t>
+          <t>Источник: доска стрима 4</t>
         </is>
       </c>
       <c r="U15" s="22" t="inlineStr">
@@ -3553,13 +3588,13 @@
     <row r="16" ht="46" customHeight="1">
       <c r="A16" s="48" t="inlineStr">
         <is>
-          <t>DQ-02</t>
-        </is>
-      </c>
-      <c r="B16" s="48" t="inlineStr"/>
+          <t>S4-02</t>
+        </is>
+      </c>
+      <c r="B16" s="48" t="n"/>
       <c r="C16" s="22" t="inlineStr">
         <is>
-          <t>Качество данных</t>
+          <t>Стрим 4</t>
         </is>
       </c>
       <c r="D16" s="22" t="inlineStr">
@@ -3569,7 +3604,7 @@
       </c>
       <c r="E16" s="22" t="inlineStr">
         <is>
-          <t>Исправления по результатам проверок (если блокер)</t>
+          <t>Задача 4.2: исправления по проверкам (если блокер)</t>
         </is>
       </c>
       <c r="F16" s="48" t="inlineStr">
@@ -3579,13 +3614,13 @@
       </c>
       <c r="G16" s="48" t="inlineStr">
         <is>
-          <t>KT-OE</t>
-        </is>
-      </c>
-      <c r="H16" s="49" t="n">
+          <t>KT-05</t>
+        </is>
+      </c>
+      <c r="H16" s="79" t="n">
         <v>46287</v>
       </c>
-      <c r="I16" s="49" t="n">
+      <c r="I16" s="79" t="n">
         <v>46305</v>
       </c>
       <c r="J16" s="50">
@@ -3594,12 +3629,12 @@
       </c>
       <c r="K16" s="22" t="inlineStr">
         <is>
-          <t>DQ (ФИО)</t>
+          <t>Участник E</t>
         </is>
       </c>
       <c r="L16" s="22" t="inlineStr">
         <is>
-          <t>Аналитик данных</t>
+          <t>Роль E</t>
         </is>
       </c>
       <c r="M16" s="51" t="n">
@@ -3607,7 +3642,7 @@
       </c>
       <c r="N16" s="22" t="inlineStr">
         <is>
-          <t>DQ-01</t>
+          <t>S4-01</t>
         </is>
       </c>
       <c r="O16" s="22" t="inlineStr">
@@ -3630,7 +3665,7 @@
       </c>
       <c r="S16" s="22" t="inlineStr">
         <is>
-          <t>Не начинать, пока DQ-01 не дал «да, блокирует»</t>
+          <t>Не начинать, пока 4.1 не дал «да, блокирует»</t>
         </is>
       </c>
       <c r="T16" s="22" t="inlineStr"/>
@@ -3691,23 +3726,23 @@
     <row r="17" ht="46" customHeight="1">
       <c r="A17" s="52" t="inlineStr">
         <is>
-          <t>GP-01</t>
-        </is>
-      </c>
-      <c r="B17" s="52" t="inlineStr"/>
+          <t>S5-01</t>
+        </is>
+      </c>
+      <c r="B17" s="52" t="n"/>
       <c r="C17" s="23" t="inlineStr">
         <is>
-          <t>Общепроектные</t>
+          <t>Стрим 5</t>
         </is>
       </c>
       <c r="D17" s="23" t="inlineStr">
         <is>
-          <t>Планирование</t>
+          <t>Подстрим 5.3</t>
         </is>
       </c>
       <c r="E17" s="23" t="inlineStr">
         <is>
-          <t>Разделение стримов после 01.09 и план передачи</t>
+          <t>Задача 5.1: разделить стримы и план передачи</t>
         </is>
       </c>
       <c r="F17" s="52" t="inlineStr">
@@ -3720,10 +3755,10 @@
           <t>KT-01</t>
         </is>
       </c>
-      <c r="H17" s="53" t="n">
+      <c r="H17" s="80" t="n">
         <v>46266</v>
       </c>
-      <c r="I17" s="53" t="n">
+      <c r="I17" s="80" t="n">
         <v>46270</v>
       </c>
       <c r="J17" s="54">
@@ -3732,12 +3767,12 @@
       </c>
       <c r="K17" s="23" t="inlineStr">
         <is>
-          <t>Я + второй ТРП</t>
+          <t>Участник A + Участник F</t>
         </is>
       </c>
       <c r="L17" s="23" t="inlineStr">
         <is>
-          <t>Два ТРП</t>
+          <t>Две роли ведения</t>
         </is>
       </c>
       <c r="M17" s="55" t="n">
@@ -3760,17 +3795,17 @@
       </c>
       <c r="S17" s="23" t="inlineStr">
         <is>
-          <t>Таблица: стрим → кто ведёт с 01.09</t>
+          <t>Таблица: стрим → кто ведёт с даты X</t>
         </is>
       </c>
       <c r="T17" s="23" t="inlineStr">
         <is>
-          <t>Этот файл, лист План_работ</t>
+          <t>Источник: этот файл</t>
         </is>
       </c>
       <c r="U17" s="23" t="inlineStr">
         <is>
-          <t>Критично, чтобы не тащить все стримы до ОЭ</t>
+          <t>Чтобы не тащить все стримы одному</t>
         </is>
       </c>
       <c r="V17" s="38">
@@ -3829,23 +3864,23 @@
     <row r="18" ht="46" customHeight="1">
       <c r="A18" s="52" t="inlineStr">
         <is>
-          <t>GP-02</t>
-        </is>
-      </c>
-      <c r="B18" s="52" t="inlineStr"/>
+          <t>S5-02</t>
+        </is>
+      </c>
+      <c r="B18" s="52" t="n"/>
       <c r="C18" s="23" t="inlineStr">
         <is>
-          <t>Общепроектные</t>
+          <t>Стрим 5</t>
         </is>
       </c>
       <c r="D18" s="23" t="inlineStr">
         <is>
-          <t>Отчётность</t>
+          <t>Подстрим 5.7</t>
         </is>
       </c>
       <c r="E18" s="23" t="inlineStr">
         <is>
-          <t>Еженедельный письменный статус вместо импровизации на дэйли</t>
+          <t>Задача 5.2: короткий письменный статус вместо длинных обсуждений</t>
         </is>
       </c>
       <c r="F18" s="52" t="inlineStr">
@@ -3858,10 +3893,10 @@
           <t>KT-01</t>
         </is>
       </c>
-      <c r="H18" s="53" t="n">
+      <c r="H18" s="80" t="n">
         <v>46258</v>
       </c>
-      <c r="I18" s="53" t="n">
+      <c r="I18" s="80" t="n">
         <v>46315</v>
       </c>
       <c r="J18" s="54">
@@ -3870,12 +3905,12 @@
       </c>
       <c r="K18" s="23" t="inlineStr">
         <is>
-          <t>Я</t>
+          <t>Участник A</t>
         </is>
       </c>
       <c r="L18" s="23" t="inlineStr">
         <is>
-          <t>ТРП</t>
+          <t>Роль A</t>
         </is>
       </c>
       <c r="M18" s="55" t="n">
@@ -3903,12 +3938,12 @@
       </c>
       <c r="T18" s="23" t="inlineStr">
         <is>
-          <t>Чат команды</t>
+          <t>Источник: чат команды</t>
         </is>
       </c>
       <c r="U18" s="23" t="inlineStr">
         <is>
-          <t>Не задача Confluence — ритуал</t>
+          <t>Ритуал, не задача доски</t>
         </is>
       </c>
       <c r="V18" s="38">
@@ -3967,23 +4002,23 @@
     <row r="19" ht="46" customHeight="1">
       <c r="A19" s="52" t="inlineStr">
         <is>
-          <t>GP-03</t>
-        </is>
-      </c>
-      <c r="B19" s="52" t="inlineStr"/>
+          <t>S5-03</t>
+        </is>
+      </c>
+      <c r="B19" s="52" t="n"/>
       <c r="C19" s="23" t="inlineStr">
         <is>
-          <t>Общепроектные</t>
+          <t>Стрим 5</t>
         </is>
       </c>
       <c r="D19" s="23" t="inlineStr">
         <is>
-          <t>Scope</t>
+          <t>Подстрим 5.6</t>
         </is>
       </c>
       <c r="E19" s="23" t="inlineStr">
         <is>
-          <t>Scope / отчётность / регламенты — только если есть срок на мне</t>
+          <t>Задача 5.3: подстримы отчётности — только при своём сроке</t>
         </is>
       </c>
       <c r="F19" s="52" t="inlineStr">
@@ -3996,10 +4031,10 @@
           <t>KT-01</t>
         </is>
       </c>
-      <c r="H19" s="53" t="n">
+      <c r="H19" s="80" t="n">
         <v>46273</v>
       </c>
-      <c r="I19" s="53" t="n">
+      <c r="I19" s="80" t="n">
         <v>46277</v>
       </c>
       <c r="J19" s="54">
@@ -4008,12 +4043,12 @@
       </c>
       <c r="K19" s="23" t="inlineStr">
         <is>
-          <t>РП / я</t>
+          <t>Участник G / Участник A</t>
         </is>
       </c>
       <c r="L19" s="23" t="inlineStr">
         <is>
-          <t>ТРП</t>
+          <t>Роль A</t>
         </is>
       </c>
       <c r="M19" s="55" t="n">
@@ -4036,17 +4071,17 @@
       </c>
       <c r="S19" s="23" t="inlineStr">
         <is>
-          <t>Просмотреть почту: есть ли дедлайн на мне. Если нет — не вести</t>
+          <t>Просмотреть входящие: есть ли дедлайн на мне. Если нет — не вести</t>
         </is>
       </c>
       <c r="T19" s="23" t="inlineStr">
         <is>
-          <t>Почта, доска</t>
+          <t>Источник: почта / доска</t>
         </is>
       </c>
       <c r="U19" s="23" t="inlineStr">
         <is>
-          <t>Не плодить 8 строк заранее</t>
+          <t>Не плодить лишние строки</t>
         </is>
       </c>
       <c r="V19" s="38">
@@ -4110,8 +4145,8 @@
       <c r="E20" s="56" t="n"/>
       <c r="F20" s="56" t="n"/>
       <c r="G20" s="56" t="n"/>
-      <c r="H20" s="57" t="n"/>
-      <c r="I20" s="57" t="n"/>
+      <c r="H20" s="81" t="n"/>
+      <c r="I20" s="81" t="n"/>
       <c r="J20" s="58">
         <f>IF(OR(H20="",I20=""),"",I20-H20+1)</f>
         <v/>
@@ -4188,8 +4223,8 @@
       <c r="E21" s="56" t="n"/>
       <c r="F21" s="56" t="n"/>
       <c r="G21" s="56" t="n"/>
-      <c r="H21" s="57" t="n"/>
-      <c r="I21" s="57" t="n"/>
+      <c r="H21" s="81" t="n"/>
+      <c r="I21" s="81" t="n"/>
       <c r="J21" s="58">
         <f>IF(OR(H21="",I21=""),"",I21-H21+1)</f>
         <v/>
@@ -4266,8 +4301,8 @@
       <c r="E22" s="56" t="n"/>
       <c r="F22" s="56" t="n"/>
       <c r="G22" s="56" t="n"/>
-      <c r="H22" s="57" t="n"/>
-      <c r="I22" s="57" t="n"/>
+      <c r="H22" s="81" t="n"/>
+      <c r="I22" s="81" t="n"/>
       <c r="J22" s="58">
         <f>IF(OR(H22="",I22=""),"",I22-H22+1)</f>
         <v/>
@@ -4344,8 +4379,8 @@
       <c r="E23" s="56" t="n"/>
       <c r="F23" s="56" t="n"/>
       <c r="G23" s="56" t="n"/>
-      <c r="H23" s="57" t="n"/>
-      <c r="I23" s="57" t="n"/>
+      <c r="H23" s="81" t="n"/>
+      <c r="I23" s="81" t="n"/>
       <c r="J23" s="58">
         <f>IF(OR(H23="",I23=""),"",I23-H23+1)</f>
         <v/>
@@ -4422,8 +4457,8 @@
       <c r="E24" s="56" t="n"/>
       <c r="F24" s="56" t="n"/>
       <c r="G24" s="56" t="n"/>
-      <c r="H24" s="57" t="n"/>
-      <c r="I24" s="57" t="n"/>
+      <c r="H24" s="81" t="n"/>
+      <c r="I24" s="81" t="n"/>
       <c r="J24" s="58">
         <f>IF(OR(H24="",I24=""),"",I24-H24+1)</f>
         <v/>
@@ -4500,8 +4535,8 @@
       <c r="E25" s="56" t="n"/>
       <c r="F25" s="56" t="n"/>
       <c r="G25" s="56" t="n"/>
-      <c r="H25" s="57" t="n"/>
-      <c r="I25" s="57" t="n"/>
+      <c r="H25" s="81" t="n"/>
+      <c r="I25" s="81" t="n"/>
       <c r="J25" s="58">
         <f>IF(OR(H25="",I25=""),"",I25-H25+1)</f>
         <v/>
@@ -4578,8 +4613,8 @@
       <c r="E26" s="56" t="n"/>
       <c r="F26" s="56" t="n"/>
       <c r="G26" s="56" t="n"/>
-      <c r="H26" s="57" t="n"/>
-      <c r="I26" s="57" t="n"/>
+      <c r="H26" s="81" t="n"/>
+      <c r="I26" s="81" t="n"/>
       <c r="J26" s="58">
         <f>IF(OR(H26="",I26=""),"",I26-H26+1)</f>
         <v/>
@@ -4656,8 +4691,8 @@
       <c r="E27" s="56" t="n"/>
       <c r="F27" s="56" t="n"/>
       <c r="G27" s="56" t="n"/>
-      <c r="H27" s="57" t="n"/>
-      <c r="I27" s="57" t="n"/>
+      <c r="H27" s="81" t="n"/>
+      <c r="I27" s="81" t="n"/>
       <c r="J27" s="58">
         <f>IF(OR(H27="",I27=""),"",I27-H27+1)</f>
         <v/>
@@ -4734,8 +4769,8 @@
       <c r="E28" s="56" t="n"/>
       <c r="F28" s="56" t="n"/>
       <c r="G28" s="56" t="n"/>
-      <c r="H28" s="57" t="n"/>
-      <c r="I28" s="57" t="n"/>
+      <c r="H28" s="81" t="n"/>
+      <c r="I28" s="81" t="n"/>
       <c r="J28" s="58">
         <f>IF(OR(H28="",I28=""),"",I28-H28+1)</f>
         <v/>
@@ -4812,8 +4847,8 @@
       <c r="E29" s="56" t="n"/>
       <c r="F29" s="56" t="n"/>
       <c r="G29" s="56" t="n"/>
-      <c r="H29" s="57" t="n"/>
-      <c r="I29" s="57" t="n"/>
+      <c r="H29" s="81" t="n"/>
+      <c r="I29" s="81" t="n"/>
       <c r="J29" s="58">
         <f>IF(OR(H29="",I29=""),"",I29-H29+1)</f>
         <v/>
@@ -4890,8 +4925,8 @@
       <c r="E30" s="56" t="n"/>
       <c r="F30" s="56" t="n"/>
       <c r="G30" s="56" t="n"/>
-      <c r="H30" s="57" t="n"/>
-      <c r="I30" s="57" t="n"/>
+      <c r="H30" s="81" t="n"/>
+      <c r="I30" s="81" t="n"/>
       <c r="J30" s="58">
         <f>IF(OR(H30="",I30=""),"",I30-H30+1)</f>
         <v/>
@@ -4968,8 +5003,8 @@
       <c r="E31" s="56" t="n"/>
       <c r="F31" s="56" t="n"/>
       <c r="G31" s="56" t="n"/>
-      <c r="H31" s="57" t="n"/>
-      <c r="I31" s="57" t="n"/>
+      <c r="H31" s="81" t="n"/>
+      <c r="I31" s="81" t="n"/>
       <c r="J31" s="58">
         <f>IF(OR(H31="",I31=""),"",I31-H31+1)</f>
         <v/>
@@ -5046,8 +5081,8 @@
       <c r="E32" s="56" t="n"/>
       <c r="F32" s="56" t="n"/>
       <c r="G32" s="56" t="n"/>
-      <c r="H32" s="57" t="n"/>
-      <c r="I32" s="57" t="n"/>
+      <c r="H32" s="81" t="n"/>
+      <c r="I32" s="81" t="n"/>
       <c r="J32" s="58">
         <f>IF(OR(H32="",I32=""),"",I32-H32+1)</f>
         <v/>
@@ -5124,8 +5159,8 @@
       <c r="E33" s="56" t="n"/>
       <c r="F33" s="56" t="n"/>
       <c r="G33" s="56" t="n"/>
-      <c r="H33" s="57" t="n"/>
-      <c r="I33" s="57" t="n"/>
+      <c r="H33" s="81" t="n"/>
+      <c r="I33" s="81" t="n"/>
       <c r="J33" s="58">
         <f>IF(OR(H33="",I33=""),"",I33-H33+1)</f>
         <v/>
@@ -5202,8 +5237,8 @@
       <c r="E34" s="56" t="n"/>
       <c r="F34" s="56" t="n"/>
       <c r="G34" s="56" t="n"/>
-      <c r="H34" s="57" t="n"/>
-      <c r="I34" s="57" t="n"/>
+      <c r="H34" s="81" t="n"/>
+      <c r="I34" s="81" t="n"/>
       <c r="J34" s="58">
         <f>IF(OR(H34="",I34=""),"",I34-H34+1)</f>
         <v/>
@@ -5280,8 +5315,8 @@
       <c r="E35" s="56" t="n"/>
       <c r="F35" s="56" t="n"/>
       <c r="G35" s="56" t="n"/>
-      <c r="H35" s="57" t="n"/>
-      <c r="I35" s="57" t="n"/>
+      <c r="H35" s="81" t="n"/>
+      <c r="I35" s="81" t="n"/>
       <c r="J35" s="58">
         <f>IF(OR(H35="",I35=""),"",I35-H35+1)</f>
         <v/>
@@ -5358,8 +5393,8 @@
       <c r="E36" s="56" t="n"/>
       <c r="F36" s="56" t="n"/>
       <c r="G36" s="56" t="n"/>
-      <c r="H36" s="57" t="n"/>
-      <c r="I36" s="57" t="n"/>
+      <c r="H36" s="81" t="n"/>
+      <c r="I36" s="81" t="n"/>
       <c r="J36" s="58">
         <f>IF(OR(H36="",I36=""),"",I36-H36+1)</f>
         <v/>
@@ -5436,8 +5471,8 @@
       <c r="E37" s="56" t="n"/>
       <c r="F37" s="56" t="n"/>
       <c r="G37" s="56" t="n"/>
-      <c r="H37" s="57" t="n"/>
-      <c r="I37" s="57" t="n"/>
+      <c r="H37" s="81" t="n"/>
+      <c r="I37" s="81" t="n"/>
       <c r="J37" s="58">
         <f>IF(OR(H37="",I37=""),"",I37-H37+1)</f>
         <v/>
@@ -5514,8 +5549,8 @@
       <c r="E38" s="56" t="n"/>
       <c r="F38" s="56" t="n"/>
       <c r="G38" s="56" t="n"/>
-      <c r="H38" s="57" t="n"/>
-      <c r="I38" s="57" t="n"/>
+      <c r="H38" s="81" t="n"/>
+      <c r="I38" s="81" t="n"/>
       <c r="J38" s="58">
         <f>IF(OR(H38="",I38=""),"",I38-H38+1)</f>
         <v/>
@@ -5592,8 +5627,8 @@
       <c r="E39" s="56" t="n"/>
       <c r="F39" s="56" t="n"/>
       <c r="G39" s="56" t="n"/>
-      <c r="H39" s="57" t="n"/>
-      <c r="I39" s="57" t="n"/>
+      <c r="H39" s="81" t="n"/>
+      <c r="I39" s="81" t="n"/>
       <c r="J39" s="58">
         <f>IF(OR(H39="",I39=""),"",I39-H39+1)</f>
         <v/>
@@ -5670,8 +5705,8 @@
       <c r="E40" s="56" t="n"/>
       <c r="F40" s="56" t="n"/>
       <c r="G40" s="56" t="n"/>
-      <c r="H40" s="57" t="n"/>
-      <c r="I40" s="57" t="n"/>
+      <c r="H40" s="81" t="n"/>
+      <c r="I40" s="81" t="n"/>
       <c r="J40" s="58">
         <f>IF(OR(H40="",I40=""),"",I40-H40+1)</f>
         <v/>
@@ -5748,64 +5783,64 @@
     <mergeCell ref="A2:U2"/>
   </mergeCells>
   <conditionalFormatting sqref="P5:P40">
-    <cfRule type="expression" priority="1" dxfId="1">
+    <cfRule type="expression" priority="18" dxfId="1">
       <formula>P5="Готово"</formula>
     </cfRule>
-    <cfRule type="expression" priority="2" dxfId="3">
+    <cfRule type="expression" priority="19" dxfId="3">
       <formula>P5="В работе"</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" dxfId="0">
+    <cfRule type="expression" priority="20" dxfId="0">
       <formula>P5="Жду"</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" dxfId="4">
+    <cfRule type="expression" priority="21" dxfId="4">
       <formula>P5="Отложено"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B5:B40">
-    <cfRule type="expression" priority="5" dxfId="5">
+    <cfRule type="expression" priority="22" dxfId="5">
       <formula>B5="★"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I5:I40">
-    <cfRule type="expression" priority="6" dxfId="2">
+    <cfRule type="expression" priority="23" dxfId="2">
       <formula>AND(I5&lt;&gt;"",I5&lt;TODAY(),P5&lt;&gt;"Готово",P5&lt;&gt;"Отложено",P5&lt;&gt;"Передано")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="V5:AH40">
-    <cfRule type="expression" priority="7" dxfId="6">
-      <formula>AND(V5="●",$C5="Архитектура")</formula>
+    <cfRule type="expression" priority="24" dxfId="6">
+      <formula>AND(V5="●",$C5="Стрим 1")</formula>
     </cfRule>
-    <cfRule type="expression" priority="8" dxfId="7">
-      <formula>AND(V5="●",$C5="Инфраструктура")</formula>
+    <cfRule type="expression" priority="26" dxfId="7">
+      <formula>AND(V5="●",$C5="Стрим 2")</formula>
     </cfRule>
-    <cfRule type="expression" priority="9" dxfId="8">
-      <formula>AND(V5="●",$C5="ИБ")</formula>
+    <cfRule type="expression" priority="28" dxfId="8">
+      <formula>AND(V5="●",$C5="Стрим 3")</formula>
     </cfRule>
-    <cfRule type="expression" priority="10" dxfId="9">
-      <formula>AND(V5="●",$C5="Качество данных")</formula>
+    <cfRule type="expression" priority="30" dxfId="9">
+      <formula>AND(V5="●",$C5="Стрим 4")</formula>
     </cfRule>
-    <cfRule type="expression" priority="11" dxfId="10">
-      <formula>AND(V5="●",$C5="Общепроектные")</formula>
+    <cfRule type="expression" priority="32" dxfId="10">
+      <formula>AND(V5="●",$C5="Стрим 5")</formula>
     </cfRule>
-    <cfRule type="expression" priority="12" dxfId="11">
+    <cfRule type="expression" priority="34" dxfId="11">
       <formula>AND(V5="●",$B5="★")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C5:C40">
-    <cfRule type="expression" priority="13" dxfId="12">
-      <formula>C5="Архитектура"</formula>
+    <cfRule type="expression" priority="25" dxfId="12">
+      <formula>C5="Стрим 1"</formula>
     </cfRule>
-    <cfRule type="expression" priority="14" dxfId="13">
-      <formula>C5="Инфраструктура"</formula>
+    <cfRule type="expression" priority="27" dxfId="13">
+      <formula>C5="Стрим 2"</formula>
     </cfRule>
-    <cfRule type="expression" priority="15" dxfId="14">
-      <formula>C5="ИБ"</formula>
+    <cfRule type="expression" priority="29" dxfId="14">
+      <formula>C5="Стрим 3"</formula>
     </cfRule>
-    <cfRule type="expression" priority="16" dxfId="15">
-      <formula>C5="Качество данных"</formula>
+    <cfRule type="expression" priority="31" dxfId="15">
+      <formula>C5="Стрим 4"</formula>
     </cfRule>
-    <cfRule type="expression" priority="17" dxfId="4">
-      <formula>C5="Общепроектные"</formula>
+    <cfRule type="expression" priority="33" dxfId="4">
+      <formula>C5="Стрим 5"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="7">
@@ -5867,7 +5902,7 @@
     <row r="2">
       <c r="A2" s="16" t="inlineStr">
         <is>
-          <t>ПРИМЕР дат. Поставьте фактические даты из проектного плана. KT-OE — якорь правой колонки «цель».</t>
+          <t>ПРИМЕР дат. KT-05 — якорь общей цели проекта.</t>
         </is>
       </c>
     </row>
@@ -5931,10 +5966,10 @@
       </c>
       <c r="C5" s="27" t="inlineStr">
         <is>
-          <t>Зафиксирован состав работ до ОЭ и разделение стримов</t>
-        </is>
-      </c>
-      <c r="D5" s="28" t="n">
+          <t>КТ 1: зафиксирован состав работ и разделение стримов</t>
+        </is>
+      </c>
+      <c r="D5" s="72" t="n">
         <v>46270</v>
       </c>
       <c r="E5" s="27" t="inlineStr">
@@ -5944,12 +5979,12 @@
       </c>
       <c r="F5" s="27" t="inlineStr">
         <is>
-          <t>Общепроектные, все ТРП</t>
+          <t>Стрим 5, роли ведения</t>
         </is>
       </c>
       <c r="G5" s="27" t="inlineStr">
         <is>
-          <t>Есть список: что закрываем к ОЭ, что после 01.09 у второго ТРП</t>
+          <t>Есть список: что закрываем к цели, что передаём</t>
         </is>
       </c>
       <c r="H5" s="62" t="inlineStr">
@@ -5959,7 +5994,7 @@
       </c>
       <c r="I5" s="27" t="inlineStr">
         <is>
-          <t>Сделать в первую неделю после выхода коллеги</t>
+          <t>Сделать после возвращения второго участника</t>
         </is>
       </c>
     </row>
@@ -5976,10 +6011,10 @@
       </c>
       <c r="C6" s="27" t="inlineStr">
         <is>
-          <t>Концептуальный дизайн согласован</t>
-        </is>
-      </c>
-      <c r="D6" s="28" t="n">
+          <t>КТ 2: документ этапа согласован</t>
+        </is>
+      </c>
+      <c r="D6" s="72" t="n">
         <v>46277</v>
       </c>
       <c r="E6" s="27" t="inlineStr">
@@ -5989,12 +6024,12 @@
       </c>
       <c r="F6" s="27" t="inlineStr">
         <is>
-          <t>Архитектура, ИБ, Инфраструктура</t>
+          <t>Стрим 1, Стрим 3, Стрим 2</t>
         </is>
       </c>
       <c r="G6" s="27" t="inlineStr">
         <is>
-          <t>Документ на общем диске, замечания либо закрыты, либо в бэклоге с датой</t>
+          <t>Документ на общем диске, замечания закрыты или в бэклоге</t>
         </is>
       </c>
       <c r="H6" s="63" t="inlineStr">
@@ -6004,7 +6039,7 @@
       </c>
       <c r="I6" s="27" t="inlineStr">
         <is>
-          <t>Вход для сетевых схем</t>
+          <t>Вход для схем</t>
         </is>
       </c>
     </row>
@@ -6021,10 +6056,10 @@
       </c>
       <c r="C7" s="27" t="inlineStr">
         <is>
-          <t>Сетевые схемы и сайзинг готовы</t>
-        </is>
-      </c>
-      <c r="D7" s="28" t="n">
+          <t>КТ 3: схемы и параметры готовы</t>
+        </is>
+      </c>
+      <c r="D7" s="72" t="n">
         <v>46291</v>
       </c>
       <c r="E7" s="27" t="inlineStr">
@@ -6034,12 +6069,12 @@
       </c>
       <c r="F7" s="27" t="inlineStr">
         <is>
-          <t>Архитектура, Инфраструктура</t>
+          <t>Стрим 1, Стрим 2</t>
         </is>
       </c>
       <c r="G7" s="27" t="inlineStr">
         <is>
-          <t>Схемы + таблица мощности согласованы с инфрой, путь в «Источник»</t>
+          <t>Схемы + таблица параметров согласованы, путь в «Источник»</t>
         </is>
       </c>
       <c r="H7" s="27" t="inlineStr">
@@ -6049,7 +6084,7 @@
       </c>
       <c r="I7" s="27" t="inlineStr">
         <is>
-          <t>Сайзинг — типичный ★ недели</t>
+          <t>Расчёт параметров — типичный ★</t>
         </is>
       </c>
     </row>
@@ -6066,10 +6101,10 @@
       </c>
       <c r="C8" s="27" t="inlineStr">
         <is>
-          <t>Допуск ИБ в ОЭ</t>
-        </is>
-      </c>
-      <c r="D8" s="28" t="n">
+          <t>КТ 4: допуск стрима 3</t>
+        </is>
+      </c>
+      <c r="D8" s="72" t="n">
         <v>46305</v>
       </c>
       <c r="E8" s="27" t="inlineStr">
@@ -6079,12 +6114,12 @@
       </c>
       <c r="F8" s="27" t="inlineStr">
         <is>
-          <t>ИБ, Архитектура, Инфраструктура</t>
+          <t>Стрим 3, Стрим 1, Стрим 2</t>
         </is>
       </c>
       <c r="G8" s="27" t="inlineStr">
         <is>
-          <t>Замечания закрыты или принят остаточный риск, есть протокол допуска</t>
+          <t>Замечания закрыты или принят остаточный риск, есть протокол</t>
         </is>
       </c>
       <c r="H8" s="27" t="inlineStr">
@@ -6094,27 +6129,27 @@
       </c>
       <c r="I8" s="27" t="inlineStr">
         <is>
-          <t>Сверять на статусах ИБ</t>
+          <t>Сверять на статусах стрима 3</t>
         </is>
       </c>
     </row>
     <row r="9" ht="48" customHeight="1">
       <c r="A9" s="64" t="inlineStr">
         <is>
-          <t>KT-OE</t>
+          <t>KT-05</t>
         </is>
       </c>
       <c r="B9" s="65" t="inlineStr">
         <is>
-          <t>Опытная эксплуатация</t>
+          <t>Цель проекта</t>
         </is>
       </c>
       <c r="C9" s="27" t="inlineStr">
         <is>
-          <t>Старт опытной эксплуатации</t>
-        </is>
-      </c>
-      <c r="D9" s="28" t="n">
+          <t>КТ 5: старт этапа проверки</t>
+        </is>
+      </c>
+      <c r="D9" s="72" t="n">
         <v>46315</v>
       </c>
       <c r="E9" s="27" t="inlineStr">
@@ -6124,12 +6159,12 @@
       </c>
       <c r="F9" s="27" t="inlineStr">
         <is>
-          <t>Архитектура, Инфраструктура, ИБ, Качество данных</t>
+          <t>Стрим 1, Стрим 2, Стрим 3, Стрим 4</t>
         </is>
       </c>
       <c r="G9" s="27" t="inlineStr">
         <is>
-          <t>Пакет артефактов + контур + допуск ИБ + решение по данным</t>
+          <t>Пакет артефактов + среда + допуск + решение по данным</t>
         </is>
       </c>
       <c r="H9" s="27" t="inlineStr">
@@ -6147,7 +6182,7 @@
       <c r="A10" s="27" t="n"/>
       <c r="B10" s="27" t="n"/>
       <c r="C10" s="27" t="n"/>
-      <c r="D10" s="66" t="n"/>
+      <c r="D10" s="82" t="n"/>
       <c r="E10" s="27" t="n"/>
       <c r="F10" s="27" t="n"/>
       <c r="G10" s="27" t="n"/>
@@ -6158,7 +6193,7 @@
       <c r="A11" s="27" t="n"/>
       <c r="B11" s="27" t="n"/>
       <c r="C11" s="27" t="n"/>
-      <c r="D11" s="66" t="n"/>
+      <c r="D11" s="82" t="n"/>
       <c r="E11" s="27" t="n"/>
       <c r="F11" s="27" t="n"/>
       <c r="G11" s="27" t="n"/>
@@ -6169,7 +6204,7 @@
       <c r="A12" s="27" t="n"/>
       <c r="B12" s="27" t="n"/>
       <c r="C12" s="27" t="n"/>
-      <c r="D12" s="66" t="n"/>
+      <c r="D12" s="82" t="n"/>
       <c r="E12" s="27" t="n"/>
       <c r="F12" s="27" t="n"/>
       <c r="G12" s="27" t="n"/>
@@ -6180,7 +6215,7 @@
       <c r="A13" s="27" t="n"/>
       <c r="B13" s="27" t="n"/>
       <c r="C13" s="27" t="n"/>
-      <c r="D13" s="66" t="n"/>
+      <c r="D13" s="82" t="n"/>
       <c r="E13" s="27" t="n"/>
       <c r="F13" s="27" t="n"/>
       <c r="G13" s="27" t="n"/>
@@ -6191,7 +6226,7 @@
       <c r="A14" s="27" t="n"/>
       <c r="B14" s="27" t="n"/>
       <c r="C14" s="27" t="n"/>
-      <c r="D14" s="66" t="n"/>
+      <c r="D14" s="82" t="n"/>
       <c r="E14" s="27" t="n"/>
       <c r="F14" s="27" t="n"/>
       <c r="G14" s="27" t="n"/>
@@ -6202,7 +6237,7 @@
       <c r="A15" s="27" t="n"/>
       <c r="B15" s="27" t="n"/>
       <c r="C15" s="27" t="n"/>
-      <c r="D15" s="66" t="n"/>
+      <c r="D15" s="82" t="n"/>
       <c r="E15" s="27" t="n"/>
       <c r="F15" s="27" t="n"/>
       <c r="G15" s="27" t="n"/>
@@ -6250,14 +6285,14 @@
     <row r="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>Бизнес-задачи и проектные цели — к ним привязывается план (колонка «Бизнес ID»)</t>
+          <t>Бизнес-задачи и цели — к ним привязывается план (колонка «Бизнес ID»)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="16" t="inlineStr">
         <is>
-          <t>ПРИМЕРЫ. Замените формулировками из устава / scope / протоколов. ID вида B-01 не меняйте в уже привязанных строках плана.</t>
+          <t>ПРИМЕРЫ. Обезличенные формулировки. ID вида B-01 не меняйте в уже привязанных строках плана.</t>
         </is>
       </c>
     </row>
@@ -6306,27 +6341,27 @@
       </c>
       <c r="B5" s="27" t="inlineStr">
         <is>
-          <t>Выход в опытную эксплуатацию</t>
+          <t>Цель 1: выход на этап проверки</t>
         </is>
       </c>
       <c r="C5" s="27" t="inlineStr">
         <is>
-          <t>Без ОЭ нет проверки контура на реальных данных и нет закрытия этапа проекта</t>
+          <t>Без цели 1 нет проверки контура и закрытия этапа</t>
         </is>
       </c>
       <c r="D5" s="27" t="inlineStr">
         <is>
-          <t>Спонсор / РП (указать ФИО)</t>
+          <t>Владелец бизнеса 1</t>
         </is>
       </c>
       <c r="E5" s="27" t="inlineStr">
         <is>
-          <t>KT-OE</t>
+          <t>KT-05</t>
         </is>
       </c>
       <c r="F5" s="27" t="inlineStr">
         <is>
-          <t>Архитектура, Инфраструктура, ИБ, Качество данных</t>
+          <t>Стрим 1, Стрим 2, Стрим 3, Стрим 4</t>
         </is>
       </c>
       <c r="G5" s="27" t="inlineStr">
@@ -6343,17 +6378,17 @@
       </c>
       <c r="B6" s="27" t="inlineStr">
         <is>
-          <t>Согласованный контур и мощность</t>
+          <t>Цель 2: согласованные параметры и среда</t>
         </is>
       </c>
       <c r="C6" s="27" t="inlineStr">
         <is>
-          <t>Иначе закупки/стенд и допуск ИБ идут вслепую, срыв сроков ОЭ</t>
+          <t>Иначе подготовка среды и допуск идут вслепую</t>
         </is>
       </c>
       <c r="D6" s="27" t="inlineStr">
         <is>
-          <t>Архитектура + Инфра</t>
+          <t>Владелец стрима 1 + стрима 2</t>
         </is>
       </c>
       <c r="E6" s="27" t="inlineStr">
@@ -6363,12 +6398,12 @@
       </c>
       <c r="F6" s="27" t="inlineStr">
         <is>
-          <t>Архитектура, Инфраструктура</t>
+          <t>Стрим 1, Стрим 2</t>
         </is>
       </c>
       <c r="G6" s="27" t="inlineStr">
         <is>
-          <t>Цепочка: концепт → сети → сайзинг</t>
+          <t>Цепочка: документ → схемы → параметры</t>
         </is>
       </c>
     </row>
@@ -6380,17 +6415,17 @@
       </c>
       <c r="B7" s="27" t="inlineStr">
         <is>
-          <t>Допуск информационной безопасности</t>
+          <t>Цель 3: допуск по требованиям стрима 3</t>
         </is>
       </c>
       <c r="C7" s="27" t="inlineStr">
         <is>
-          <t>Без допуска контур нельзя выводить в ОЭ</t>
+          <t>Без допуска контур нельзя выводить на цель 1</t>
         </is>
       </c>
       <c r="D7" s="27" t="inlineStr">
         <is>
-          <t>ИБ (указать ФИО)</t>
+          <t>Владелец стрима 3</t>
         </is>
       </c>
       <c r="E7" s="27" t="inlineStr">
@@ -6400,12 +6435,12 @@
       </c>
       <c r="F7" s="27" t="inlineStr">
         <is>
-          <t>ИБ, Архитектура</t>
+          <t>Стрим 3, Стрим 1</t>
         </is>
       </c>
       <c r="G7" s="27" t="inlineStr">
         <is>
-          <t>Статусные встречи ИБ = сверка этого пункта</t>
+          <t>Статусные встречи стрима 3 = сверка</t>
         </is>
       </c>
     </row>
@@ -6417,32 +6452,32 @@
       </c>
       <c r="B8" s="27" t="inlineStr">
         <is>
-          <t>Данные пригодны для ОЭ</t>
+          <t>Цель 4: данные пригодны для проверки</t>
         </is>
       </c>
       <c r="C8" s="27" t="inlineStr">
         <is>
-          <t>ОЭ на грязных данных даёт ложный результат приёмки</t>
+          <t>Проверка на некачественных данных даёт ложный результат</t>
         </is>
       </c>
       <c r="D8" s="27" t="inlineStr">
         <is>
-          <t>Качество данных</t>
+          <t>Владелец стрима 4</t>
         </is>
       </c>
       <c r="E8" s="27" t="inlineStr">
         <is>
-          <t>KT-OE</t>
+          <t>KT-05</t>
         </is>
       </c>
       <c r="F8" s="27" t="inlineStr">
         <is>
-          <t>Качество данных</t>
+          <t>Стрим 4</t>
         </is>
       </c>
       <c r="G8" s="27" t="inlineStr">
         <is>
-          <t>Вести в плане, только если реально блокирует ОЭ</t>
+          <t>Вести только если реально блокирует цель 1</t>
         </is>
       </c>
     </row>
@@ -6454,17 +6489,17 @@
       </c>
       <c r="B9" s="27" t="inlineStr">
         <is>
-          <t>Управляемость проекта (план, scope, отчётность, регламенты)</t>
+          <t>Цель 5: управляемость проекта</t>
         </is>
       </c>
       <c r="C9" s="27" t="inlineStr">
         <is>
-          <t>Без этого дэйли превращается в разбор 30 задач без порядка</t>
+          <t>Без этого ежедневный статус превращается в разбор 30 задач без порядка</t>
         </is>
       </c>
       <c r="D9" s="27" t="inlineStr">
         <is>
-          <t>РП / ТРП</t>
+          <t>Владелец проекта / роль ведения</t>
         </is>
       </c>
       <c r="E9" s="27" t="inlineStr">
@@ -6474,12 +6509,12 @@
       </c>
       <c r="F9" s="27" t="inlineStr">
         <is>
-          <t>Общепроектные</t>
+          <t>Стрим 5</t>
         </is>
       </c>
       <c r="G9" s="27" t="inlineStr">
         <is>
-          <t>Не расписывать 8 веток, если нет вашего срока</t>
+          <t>Не расписывать все подстримы заранее</t>
         </is>
       </c>
     </row>
@@ -6577,7 +6612,7 @@
     <row r="2">
       <c r="A2" s="16" t="inlineStr">
         <is>
-          <t>Тип ОН = нельзя начать, пока не закончена предыдущая. НН = можно стартовать параллельно. Критичная = срыв тянет КТ/ОЭ.</t>
+          <t>Тип ОН = нельзя начать, пока не закончена предыдущая. НН = можно стартовать параллельно. Критичная = срыв тянет КТ/цель.</t>
         </is>
       </c>
     </row>
@@ -6609,7 +6644,7 @@
       </c>
       <c r="F4" s="17" t="inlineStr">
         <is>
-          <t>Критичная для ОЭ</t>
+          <t>Критичная для цель</t>
         </is>
       </c>
       <c r="G4" s="17" t="inlineStr">
@@ -6621,22 +6656,22 @@
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="19" t="inlineStr">
         <is>
-          <t>A-01</t>
+          <t>S1-01</t>
         </is>
       </c>
       <c r="B5" s="27" t="inlineStr">
         <is>
-          <t>Концепт</t>
+          <t>Задача 1.1</t>
         </is>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>
-          <t>A-02</t>
+          <t>S1-02</t>
         </is>
       </c>
       <c r="D5" s="27" t="inlineStr">
         <is>
-          <t>Сетевые схемы</t>
+          <t>Задача 1.2</t>
         </is>
       </c>
       <c r="E5" s="27" t="inlineStr">
@@ -6651,29 +6686,29 @@
       </c>
       <c r="G5" s="27" t="inlineStr">
         <is>
-          <t>Схемы без концепта — рисование в пустоту</t>
+          <t>Схемы без документа — работа в пустоту</t>
         </is>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1">
       <c r="A6" s="19" t="inlineStr">
         <is>
-          <t>A-01</t>
+          <t>S1-01</t>
         </is>
       </c>
       <c r="B6" s="27" t="inlineStr">
         <is>
-          <t>Концепт</t>
+          <t>Задача 1.1</t>
         </is>
       </c>
       <c r="C6" s="19" t="inlineStr">
         <is>
-          <t>I-01</t>
+          <t>S2-01</t>
         </is>
       </c>
       <c r="D6" s="27" t="inlineStr">
         <is>
-          <t>Требования к контуру</t>
+          <t>Задача 2.1</t>
         </is>
       </c>
       <c r="E6" s="27" t="inlineStr">
@@ -6688,29 +6723,29 @@
       </c>
       <c r="G6" s="27" t="inlineStr">
         <is>
-          <t>Инфра может готовить вопросы, не дожидаясь финала</t>
+          <t>Стрим 2 может готовить вопросы параллельно</t>
         </is>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>A-02</t>
+          <t>S1-02</t>
         </is>
       </c>
       <c r="B7" s="27" t="inlineStr">
         <is>
-          <t>Сетевые схемы</t>
+          <t>Задача 1.2</t>
         </is>
       </c>
       <c r="C7" s="19" t="inlineStr">
         <is>
-          <t>A-03</t>
+          <t>S1-03</t>
         </is>
       </c>
       <c r="D7" s="27" t="inlineStr">
         <is>
-          <t>Сайзинг</t>
+          <t>Задача 1.3</t>
         </is>
       </c>
       <c r="E7" s="27" t="inlineStr">
@@ -6725,29 +6760,29 @@
       </c>
       <c r="G7" s="27" t="inlineStr">
         <is>
-          <t>Мощность считается по зонам со схем</t>
+          <t>Параметры считаются по схемам</t>
         </is>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="19" t="inlineStr">
         <is>
-          <t>A-03</t>
+          <t>S1-03</t>
         </is>
       </c>
       <c r="B8" s="27" t="inlineStr">
         <is>
-          <t>Сайзинг</t>
+          <t>Задача 1.3</t>
         </is>
       </c>
       <c r="C8" s="19" t="inlineStr">
         <is>
-          <t>I-02</t>
+          <t>S2-02</t>
         </is>
       </c>
       <c r="D8" s="27" t="inlineStr">
         <is>
-          <t>Стенд</t>
+          <t>Задача 2.2</t>
         </is>
       </c>
       <c r="E8" s="27" t="inlineStr">
@@ -6762,29 +6797,29 @@
       </c>
       <c r="G8" s="27" t="inlineStr">
         <is>
-          <t>Иначе стенд могут собрать «не того размера»</t>
+          <t>Иначе среда может быть собрана «не того размера»</t>
         </is>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1">
       <c r="A9" s="19" t="inlineStr">
         <is>
-          <t>A-01</t>
+          <t>S1-01</t>
         </is>
       </c>
       <c r="B9" s="27" t="inlineStr">
         <is>
-          <t>Концепт</t>
+          <t>Задача 1.1</t>
         </is>
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t>IB-02</t>
+          <t>S3-02</t>
         </is>
       </c>
       <c r="D9" s="27" t="inlineStr">
         <is>
-          <t>Замечания ИБ</t>
+          <t>Задача 3.2</t>
         </is>
       </c>
       <c r="E9" s="27" t="inlineStr">
@@ -6799,29 +6834,29 @@
       </c>
       <c r="G9" s="27" t="inlineStr">
         <is>
-          <t>ИБ комментирует документ и схемы</t>
+          <t>Стрим 3 комментирует документ и схемы</t>
         </is>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1">
       <c r="A10" s="19" t="inlineStr">
         <is>
-          <t>A-02</t>
+          <t>S1-02</t>
         </is>
       </c>
       <c r="B10" s="27" t="inlineStr">
         <is>
-          <t>Сетевые схемы</t>
+          <t>Задача 1.2</t>
         </is>
       </c>
       <c r="C10" s="19" t="inlineStr">
         <is>
-          <t>IB-02</t>
+          <t>S3-02</t>
         </is>
       </c>
       <c r="D10" s="27" t="inlineStr">
         <is>
-          <t>Замечания ИБ</t>
+          <t>Задача 3.2</t>
         </is>
       </c>
       <c r="E10" s="27" t="inlineStr">
@@ -6836,29 +6871,29 @@
       </c>
       <c r="G10" s="27" t="inlineStr">
         <is>
-          <t>Сегментация / периметр</t>
+          <t>Проверка сегментации / границ</t>
         </is>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1">
       <c r="A11" s="19" t="inlineStr">
         <is>
-          <t>IB-01</t>
+          <t>S3-01</t>
         </is>
       </c>
       <c r="B11" s="27" t="inlineStr">
         <is>
-          <t>Реестр ИБ</t>
+          <t>Задача 3.1</t>
         </is>
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t>IB-02</t>
+          <t>S3-02</t>
         </is>
       </c>
       <c r="D11" s="27" t="inlineStr">
         <is>
-          <t>Закрытие замечаний</t>
+          <t>Задача 3.2</t>
         </is>
       </c>
       <c r="E11" s="27" t="inlineStr">
@@ -6873,29 +6908,29 @@
       </c>
       <c r="G11" s="27" t="inlineStr">
         <is>
-          <t>Сначала понятный список, потом закрытие</t>
+          <t>Сначала список, потом закрытие</t>
         </is>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1">
       <c r="A12" s="19" t="inlineStr">
         <is>
-          <t>IB-02</t>
+          <t>S3-02</t>
         </is>
       </c>
       <c r="B12" s="27" t="inlineStr">
         <is>
-          <t>Замечания ИБ</t>
+          <t>Задача 3.2</t>
         </is>
       </c>
       <c r="C12" s="19" t="inlineStr">
         <is>
-          <t>IB-03</t>
+          <t>S3-03</t>
         </is>
       </c>
       <c r="D12" s="27" t="inlineStr">
         <is>
-          <t>Допуск</t>
+          <t>Задача 3.3</t>
         </is>
       </c>
       <c r="E12" s="27" t="inlineStr">
@@ -6910,29 +6945,29 @@
       </c>
       <c r="G12" s="27" t="inlineStr">
         <is>
-          <t>Допуск = закрытый (или принятый) остаток</t>
+          <t>Допуск = закрытый или принятый остаток</t>
         </is>
       </c>
     </row>
     <row r="13" ht="32" customHeight="1">
       <c r="A13" s="19" t="inlineStr">
         <is>
-          <t>I-02</t>
+          <t>S2-02</t>
         </is>
       </c>
       <c r="B13" s="27" t="inlineStr">
         <is>
-          <t>Стенд</t>
+          <t>Задача 2.2</t>
         </is>
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>IB-03</t>
+          <t>S3-03</t>
         </is>
       </c>
       <c r="D13" s="27" t="inlineStr">
         <is>
-          <t>Допуск</t>
+          <t>Задача 3.3</t>
         </is>
       </c>
       <c r="E13" s="27" t="inlineStr">
@@ -6947,29 +6982,29 @@
       </c>
       <c r="G13" s="27" t="inlineStr">
         <is>
-          <t>Допускают конкретный контур, не бумагу</t>
+          <t>Допускают конкретную среду, не только бумагу</t>
         </is>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1">
       <c r="A14" s="19" t="inlineStr">
         <is>
-          <t>I-02</t>
+          <t>S2-02</t>
         </is>
       </c>
       <c r="B14" s="27" t="inlineStr">
         <is>
-          <t>Стенд</t>
+          <t>Задача 2.2</t>
         </is>
       </c>
       <c r="C14" s="19" t="inlineStr">
         <is>
-          <t>I-03</t>
+          <t>S2-03</t>
         </is>
       </c>
       <c r="D14" s="27" t="inlineStr">
         <is>
-          <t>Готовность инфры</t>
+          <t>Задача 2.3</t>
         </is>
       </c>
       <c r="E14" s="27" t="inlineStr">
@@ -6984,29 +7019,29 @@
       </c>
       <c r="G14" s="27" t="inlineStr">
         <is>
-          <t>Чеклист после появления стенда</t>
+          <t>Чеклист после появления среды</t>
         </is>
       </c>
     </row>
     <row r="15" ht="32" customHeight="1">
       <c r="A15" s="19" t="inlineStr">
         <is>
-          <t>A-04</t>
+          <t>S1-04</t>
         </is>
       </c>
       <c r="B15" s="27" t="inlineStr">
         <is>
-          <t>Пакет арх</t>
+          <t>Задача 1.4</t>
         </is>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>KT-OE</t>
+          <t>KT-05</t>
         </is>
       </c>
       <c r="D15" s="27" t="inlineStr">
         <is>
-          <t>Старт ОЭ</t>
+          <t>КТ 5 / цель</t>
         </is>
       </c>
       <c r="E15" s="27" t="inlineStr">
@@ -7021,29 +7056,29 @@
       </c>
       <c r="G15" s="27" t="inlineStr">
         <is>
-          <t>Артефакты в пакете ОЭ</t>
+          <t>Артефакты в пакете цели</t>
         </is>
       </c>
     </row>
     <row r="16" ht="32" customHeight="1">
       <c r="A16" s="19" t="inlineStr">
         <is>
-          <t>I-03</t>
+          <t>S2-03</t>
         </is>
       </c>
       <c r="B16" s="27" t="inlineStr">
         <is>
-          <t>Готовность инфры</t>
+          <t>Задача 2.3</t>
         </is>
       </c>
       <c r="C16" s="19" t="inlineStr">
         <is>
-          <t>KT-OE</t>
+          <t>KT-05</t>
         </is>
       </c>
       <c r="D16" s="27" t="inlineStr">
         <is>
-          <t>Старт ОЭ</t>
+          <t>КТ 5 / цель</t>
         </is>
       </c>
       <c r="E16" s="27" t="inlineStr">
@@ -7058,29 +7093,29 @@
       </c>
       <c r="G16" s="27" t="inlineStr">
         <is>
-          <t>Контур живой</t>
+          <t>Среда готова</t>
         </is>
       </c>
     </row>
     <row r="17" ht="32" customHeight="1">
       <c r="A17" s="19" t="inlineStr">
         <is>
-          <t>IB-03</t>
+          <t>S3-03</t>
         </is>
       </c>
       <c r="B17" s="27" t="inlineStr">
         <is>
-          <t>Допуск ИБ</t>
+          <t>Задача 3.3</t>
         </is>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>KT-OE</t>
+          <t>KT-05</t>
         </is>
       </c>
       <c r="D17" s="27" t="inlineStr">
         <is>
-          <t>Старт ОЭ</t>
+          <t>КТ 5 / цель</t>
         </is>
       </c>
       <c r="E17" s="27" t="inlineStr">
@@ -7095,29 +7130,29 @@
       </c>
       <c r="G17" s="27" t="inlineStr">
         <is>
-          <t>Без допуска ОЭ нельзя</t>
+          <t>Без допуска цель нельзя</t>
         </is>
       </c>
     </row>
     <row r="18" ht="32" customHeight="1">
       <c r="A18" s="19" t="inlineStr">
         <is>
-          <t>DQ-01</t>
+          <t>S4-01</t>
         </is>
       </c>
       <c r="B18" s="27" t="inlineStr">
         <is>
-          <t>Нужны ли проверки</t>
+          <t>Задача 4.1</t>
         </is>
       </c>
       <c r="C18" s="19" t="inlineStr">
         <is>
-          <t>DQ-02</t>
+          <t>S4-02</t>
         </is>
       </c>
       <c r="D18" s="27" t="inlineStr">
         <is>
-          <t>Исправления</t>
+          <t>Задача 4.2</t>
         </is>
       </c>
       <c r="E18" s="27" t="inlineStr">
@@ -7132,29 +7167,29 @@
       </c>
       <c r="G18" s="27" t="inlineStr">
         <is>
-          <t>Только если DQ-01 = да, блокер</t>
+          <t>Только если 4.1 = да, блокер</t>
         </is>
       </c>
     </row>
     <row r="19" ht="32" customHeight="1">
       <c r="A19" s="19" t="inlineStr">
         <is>
-          <t>GP-01</t>
+          <t>S5-01</t>
         </is>
       </c>
       <c r="B19" s="27" t="inlineStr">
         <is>
-          <t>Разделение стримов 01.09</t>
+          <t>Задача 5.1</t>
         </is>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>A-03</t>
+          <t>S1-03</t>
         </is>
       </c>
       <c r="D19" s="27" t="inlineStr">
         <is>
-          <t>Сайзинг и дальше</t>
+          <t>Задача 1.3 и дальше</t>
         </is>
       </c>
       <c r="E19" s="27" t="inlineStr">
@@ -7169,7 +7204,7 @@
       </c>
       <c r="G19" s="27" t="inlineStr">
         <is>
-          <t>Иначе вы тащите все стримы и срываете передачу</t>
+          <t>Иначе один участник тащит все стримы</t>
         </is>
       </c>
     </row>
@@ -7288,14 +7323,14 @@
     <row r="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>Ресурсы: люди, стенды, внешние. Связь с задачами плана по ID.</t>
+          <t>Ресурсы: люди, среды, внешние. Связь с задачами плана по ID.</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="16" t="inlineStr">
         <is>
-          <t>Загрузка &gt;100% на одной неделе = конфликт. Второй ТРП до 01.09 в отпуске — это уже отражено.</t>
+          <t>Загрузка &gt;100% на одной неделе = конфликт. Временное покрытие чужих стримов отражено отдельной строкой.</t>
         </is>
       </c>
     </row>
@@ -7307,7 +7342,7 @@
       </c>
       <c r="B4" s="17" t="inlineStr">
         <is>
-          <t>ФИО / название</t>
+          <t>Имя / название</t>
         </is>
       </c>
       <c r="C4" s="17" t="inlineStr">
@@ -7354,7 +7389,7 @@
       </c>
       <c r="B5" s="27" t="inlineStr">
         <is>
-          <t>Я (ТРП)</t>
+          <t>Участник A</t>
         </is>
       </c>
       <c r="C5" s="27" t="inlineStr">
@@ -7364,18 +7399,18 @@
       </c>
       <c r="D5" s="27" t="inlineStr">
         <is>
-          <t>Архитектура</t>
+          <t>Стрим 1</t>
         </is>
       </c>
       <c r="E5" s="27" t="inlineStr">
         <is>
-          <t>Ведение стрима, концепт, сайзинг, пакет ОЭ</t>
-        </is>
-      </c>
-      <c r="F5" s="28" t="n">
+          <t>Ведение стрима 1, документ, параметры, пакет</t>
+        </is>
+      </c>
+      <c r="F5" s="72" t="n">
         <v>46258</v>
       </c>
-      <c r="G5" s="28" t="n">
+      <c r="G5" s="72" t="n">
         <v>46315</v>
       </c>
       <c r="H5" s="67" t="n">
@@ -7383,7 +7418,7 @@
       </c>
       <c r="I5" s="27" t="inlineStr">
         <is>
-          <t>A-01,A-03,A-04,IB-01,GP-01</t>
+          <t>S1-01,S1-03,S1-04,S3-01,S5-01</t>
         </is>
       </c>
     </row>
@@ -7395,7 +7430,7 @@
       </c>
       <c r="B6" s="27" t="inlineStr">
         <is>
-          <t>Я (ТРП) — покрытие чужих стримов</t>
+          <t>Участник A — временное покрытие</t>
         </is>
       </c>
       <c r="C6" s="27" t="inlineStr">
@@ -7405,18 +7440,18 @@
       </c>
       <c r="D6" s="27" t="inlineStr">
         <is>
-          <t>Общепроектные</t>
+          <t>Стрим 5</t>
         </is>
       </c>
       <c r="E6" s="27" t="inlineStr">
         <is>
-          <t>Временно все стримы до 01.09</t>
-        </is>
-      </c>
-      <c r="F6" s="28" t="n">
+          <t>Временно несколько стримов до даты X</t>
+        </is>
+      </c>
+      <c r="F6" s="72" t="n">
         <v>46258</v>
       </c>
-      <c r="G6" s="28" t="n">
+      <c r="G6" s="72" t="n">
         <v>46266</v>
       </c>
       <c r="H6" s="68" t="n">
@@ -7424,7 +7459,7 @@
       </c>
       <c r="I6" s="27" t="inlineStr">
         <is>
-          <t>IB-01,GP-02</t>
+          <t>S3-01,S5-02</t>
         </is>
       </c>
     </row>
@@ -7436,7 +7471,7 @@
       </c>
       <c r="B7" s="27" t="inlineStr">
         <is>
-          <t>Второй ТРП (ФИО)</t>
+          <t>Участник F</t>
         </is>
       </c>
       <c r="C7" s="27" t="inlineStr">
@@ -7446,18 +7481,18 @@
       </c>
       <c r="D7" s="27" t="inlineStr">
         <is>
-          <t>Общепроектные</t>
+          <t>Стрим 5</t>
         </is>
       </c>
       <c r="E7" s="27" t="inlineStr">
         <is>
-          <t>Возврат стримов с 01.09</t>
-        </is>
-      </c>
-      <c r="F7" s="28" t="n">
+          <t>Возврат стримов с даты X</t>
+        </is>
+      </c>
+      <c r="F7" s="72" t="n">
         <v>46266</v>
       </c>
-      <c r="G7" s="28" t="n">
+      <c r="G7" s="72" t="n">
         <v>46315</v>
       </c>
       <c r="H7" s="67" t="n">
@@ -7465,7 +7500,7 @@
       </c>
       <c r="I7" s="27" t="inlineStr">
         <is>
-          <t>GP-01</t>
+          <t>S5-01</t>
         </is>
       </c>
     </row>
@@ -7477,7 +7512,7 @@
       </c>
       <c r="B8" s="27" t="inlineStr">
         <is>
-          <t>Инженер инфраструктуры (ФИО)</t>
+          <t>Участник C</t>
         </is>
       </c>
       <c r="C8" s="27" t="inlineStr">
@@ -7487,18 +7522,18 @@
       </c>
       <c r="D8" s="27" t="inlineStr">
         <is>
-          <t>Инфраструктура</t>
+          <t>Стрим 2</t>
         </is>
       </c>
       <c r="E8" s="27" t="inlineStr">
         <is>
-          <t>Контур, стенд, готовность</t>
-        </is>
-      </c>
-      <c r="F8" s="28" t="n">
+          <t>Среда, стенд, готовность</t>
+        </is>
+      </c>
+      <c r="F8" s="72" t="n">
         <v>46265</v>
       </c>
-      <c r="G8" s="28" t="n">
+      <c r="G8" s="72" t="n">
         <v>46315</v>
       </c>
       <c r="H8" s="67" t="n">
@@ -7506,7 +7541,7 @@
       </c>
       <c r="I8" s="27" t="inlineStr">
         <is>
-          <t>I-01,I-02,I-03</t>
+          <t>S2-01,S2-02,S2-03</t>
         </is>
       </c>
     </row>
@@ -7518,7 +7553,7 @@
       </c>
       <c r="B9" s="27" t="inlineStr">
         <is>
-          <t>Стенд / контур ОЭ</t>
+          <t>Среда / стенд цели</t>
         </is>
       </c>
       <c r="C9" s="27" t="inlineStr">
@@ -7528,18 +7563,18 @@
       </c>
       <c r="D9" s="27" t="inlineStr">
         <is>
-          <t>Инфраструктура</t>
+          <t>Стрим 2</t>
         </is>
       </c>
       <c r="E9" s="27" t="inlineStr">
         <is>
-          <t>Среда опытной эксплуатации</t>
-        </is>
-      </c>
-      <c r="F9" s="28" t="n">
+          <t>Среда этапа проверки</t>
+        </is>
+      </c>
+      <c r="F9" s="72" t="n">
         <v>46279</v>
       </c>
-      <c r="G9" s="28" t="n">
+      <c r="G9" s="72" t="n">
         <v>46315</v>
       </c>
       <c r="H9" s="68" t="n">
@@ -7547,7 +7582,7 @@
       </c>
       <c r="I9" s="27" t="inlineStr">
         <is>
-          <t>I-02,I-03,IB-03</t>
+          <t>S2-02,S2-03,S3-03</t>
         </is>
       </c>
     </row>
@@ -7559,7 +7594,7 @@
       </c>
       <c r="B10" s="27" t="inlineStr">
         <is>
-          <t>ИБ (ФИО)</t>
+          <t>Участник D</t>
         </is>
       </c>
       <c r="C10" s="27" t="inlineStr">
@@ -7569,7 +7604,7 @@
       </c>
       <c r="D10" s="27" t="inlineStr">
         <is>
-          <t>ИБ</t>
+          <t>Стрим 3</t>
         </is>
       </c>
       <c r="E10" s="27" t="inlineStr">
@@ -7577,10 +7612,10 @@
           <t>Замечания, статусы, допуск</t>
         </is>
       </c>
-      <c r="F10" s="28" t="n">
+      <c r="F10" s="72" t="n">
         <v>46258</v>
       </c>
-      <c r="G10" s="28" t="n">
+      <c r="G10" s="72" t="n">
         <v>46305</v>
       </c>
       <c r="H10" s="67" t="n">
@@ -7588,7 +7623,7 @@
       </c>
       <c r="I10" s="27" t="inlineStr">
         <is>
-          <t>IB-01,IB-02,IB-03</t>
+          <t>S3-01,S3-02,S3-03</t>
         </is>
       </c>
     </row>
@@ -7600,7 +7635,7 @@
       </c>
       <c r="B11" s="27" t="inlineStr">
         <is>
-          <t>Сетевой архитектор (ФИО)</t>
+          <t>Участник B</t>
         </is>
       </c>
       <c r="C11" s="27" t="inlineStr">
@@ -7610,18 +7645,18 @@
       </c>
       <c r="D11" s="27" t="inlineStr">
         <is>
-          <t>Архитектура</t>
+          <t>Стрим 1</t>
         </is>
       </c>
       <c r="E11" s="27" t="inlineStr">
         <is>
-          <t>Сетевые схемы</t>
-        </is>
-      </c>
-      <c r="F11" s="28" t="n">
+          <t>Схемы этапа</t>
+        </is>
+      </c>
+      <c r="F11" s="72" t="n">
         <v>46273</v>
       </c>
-      <c r="G11" s="28" t="n">
+      <c r="G11" s="72" t="n">
         <v>46284</v>
       </c>
       <c r="H11" s="67" t="n">
@@ -7629,7 +7664,7 @@
       </c>
       <c r="I11" s="27" t="inlineStr">
         <is>
-          <t>A-02</t>
+          <t>S1-02</t>
         </is>
       </c>
     </row>
@@ -7641,7 +7676,7 @@
       </c>
       <c r="B12" s="27" t="inlineStr">
         <is>
-          <t>Аналитик качества данных (ФИО)</t>
+          <t>Участник E</t>
         </is>
       </c>
       <c r="C12" s="27" t="inlineStr">
@@ -7651,18 +7686,18 @@
       </c>
       <c r="D12" s="27" t="inlineStr">
         <is>
-          <t>Качество данных</t>
+          <t>Стрим 4</t>
         </is>
       </c>
       <c r="E12" s="27" t="inlineStr">
         <is>
-          <t>Проверки к ОЭ</t>
-        </is>
-      </c>
-      <c r="F12" s="28" t="n">
+          <t>Проверки к цели</t>
+        </is>
+      </c>
+      <c r="F12" s="72" t="n">
         <v>46280</v>
       </c>
-      <c r="G12" s="28" t="n">
+      <c r="G12" s="72" t="n">
         <v>46305</v>
       </c>
       <c r="H12" s="67" t="n">
@@ -7670,7 +7705,7 @@
       </c>
       <c r="I12" s="27" t="inlineStr">
         <is>
-          <t>DQ-01,DQ-02</t>
+          <t>S4-01,S4-02</t>
         </is>
       </c>
     </row>
@@ -7680,8 +7715,8 @@
       <c r="C13" s="27" t="n"/>
       <c r="D13" s="27" t="n"/>
       <c r="E13" s="27" t="n"/>
-      <c r="F13" s="66" t="n"/>
-      <c r="G13" s="66" t="n"/>
+      <c r="F13" s="82" t="n"/>
+      <c r="G13" s="82" t="n"/>
       <c r="H13" s="69" t="n"/>
       <c r="I13" s="27" t="n"/>
     </row>
@@ -7691,8 +7726,8 @@
       <c r="C14" s="27" t="n"/>
       <c r="D14" s="27" t="n"/>
       <c r="E14" s="27" t="n"/>
-      <c r="F14" s="66" t="n"/>
-      <c r="G14" s="66" t="n"/>
+      <c r="F14" s="82" t="n"/>
+      <c r="G14" s="82" t="n"/>
       <c r="H14" s="69" t="n"/>
       <c r="I14" s="27" t="n"/>
     </row>
@@ -7702,8 +7737,8 @@
       <c r="C15" s="27" t="n"/>
       <c r="D15" s="27" t="n"/>
       <c r="E15" s="27" t="n"/>
-      <c r="F15" s="66" t="n"/>
-      <c r="G15" s="66" t="n"/>
+      <c r="F15" s="82" t="n"/>
+      <c r="G15" s="82" t="n"/>
       <c r="H15" s="69" t="n"/>
       <c r="I15" s="27" t="n"/>
     </row>
@@ -7713,8 +7748,8 @@
       <c r="C16" s="27" t="n"/>
       <c r="D16" s="27" t="n"/>
       <c r="E16" s="27" t="n"/>
-      <c r="F16" s="66" t="n"/>
-      <c r="G16" s="66" t="n"/>
+      <c r="F16" s="82" t="n"/>
+      <c r="G16" s="82" t="n"/>
       <c r="H16" s="69" t="n"/>
       <c r="I16" s="27" t="n"/>
     </row>
@@ -7724,8 +7759,8 @@
       <c r="C17" s="27" t="n"/>
       <c r="D17" s="27" t="n"/>
       <c r="E17" s="27" t="n"/>
-      <c r="F17" s="66" t="n"/>
-      <c r="G17" s="66" t="n"/>
+      <c r="F17" s="82" t="n"/>
+      <c r="G17" s="82" t="n"/>
       <c r="H17" s="69" t="n"/>
       <c r="I17" s="27" t="n"/>
     </row>
@@ -7735,8 +7770,8 @@
       <c r="C18" s="27" t="n"/>
       <c r="D18" s="27" t="n"/>
       <c r="E18" s="27" t="n"/>
-      <c r="F18" s="66" t="n"/>
-      <c r="G18" s="66" t="n"/>
+      <c r="F18" s="82" t="n"/>
+      <c r="G18" s="82" t="n"/>
       <c r="H18" s="69" t="n"/>
       <c r="I18" s="27" t="n"/>
     </row>
@@ -7746,8 +7781,8 @@
       <c r="C19" s="27" t="n"/>
       <c r="D19" s="27" t="n"/>
       <c r="E19" s="27" t="n"/>
-      <c r="F19" s="66" t="n"/>
-      <c r="G19" s="66" t="n"/>
+      <c r="F19" s="82" t="n"/>
+      <c r="G19" s="82" t="n"/>
       <c r="H19" s="69" t="n"/>
       <c r="I19" s="27" t="n"/>
     </row>
@@ -7834,7 +7869,7 @@
     <row r="2">
       <c r="A2" s="70" t="inlineStr">
         <is>
-          <t>Архитектура</t>
+          <t>Стрим 1</t>
         </is>
       </c>
       <c r="B2" s="70" t="inlineStr">
@@ -7876,12 +7911,12 @@
     <row r="3">
       <c r="A3" s="70" t="inlineStr">
         <is>
-          <t>Инфраструктура</t>
+          <t>Стрим 2</t>
         </is>
       </c>
       <c r="B3" s="70" t="inlineStr">
         <is>
-          <t>Финансы</t>
+          <t>Подстрим 5.1</t>
         </is>
       </c>
       <c r="C3" s="70" t="inlineStr">
@@ -7918,12 +7953,12 @@
     <row r="4">
       <c r="A4" s="70" t="inlineStr">
         <is>
-          <t>ИБ</t>
+          <t>Стрим 3</t>
         </is>
       </c>
       <c r="B4" s="70" t="inlineStr">
         <is>
-          <t>Ресурсы</t>
+          <t>Подстрим 5.2</t>
         </is>
       </c>
       <c r="C4" s="70" t="inlineStr">
@@ -7939,7 +7974,7 @@
       </c>
       <c r="F4" s="70" t="inlineStr">
         <is>
-          <t>Опытная эксплуатация</t>
+          <t>Цель проекта</t>
         </is>
       </c>
       <c r="G4" s="70" t="inlineStr">
@@ -7956,12 +7991,12 @@
     <row r="5">
       <c r="A5" s="70" t="inlineStr">
         <is>
-          <t>Качество данных</t>
+          <t>Стрим 4</t>
         </is>
       </c>
       <c r="B5" s="70" t="inlineStr">
         <is>
-          <t>Планирование</t>
+          <t>Подстрим 5.3</t>
         </is>
       </c>
       <c r="C5" s="70" t="inlineStr">
@@ -7986,12 +8021,12 @@
     <row r="6">
       <c r="A6" s="70" t="inlineStr">
         <is>
-          <t>Общепроектные</t>
+          <t>Стрим 5</t>
         </is>
       </c>
       <c r="B6" s="70" t="inlineStr">
         <is>
-          <t>Обучение</t>
+          <t>Подстрим 5.4</t>
         </is>
       </c>
       <c r="C6" s="70" t="inlineStr">
@@ -8013,7 +8048,7 @@
       <c r="A7" s="70" t="n"/>
       <c r="B7" s="70" t="inlineStr">
         <is>
-          <t>Закупки</t>
+          <t>Подстрим 5.5</t>
         </is>
       </c>
       <c r="C7" s="70" t="inlineStr">
@@ -8031,7 +8066,7 @@
       <c r="A8" s="70" t="n"/>
       <c r="B8" s="70" t="inlineStr">
         <is>
-          <t>Scope</t>
+          <t>Подстрим 5.6</t>
         </is>
       </c>
       <c r="C8" s="70" t="n"/>
@@ -8045,7 +8080,7 @@
       <c r="A9" s="70" t="n"/>
       <c r="B9" s="70" t="inlineStr">
         <is>
-          <t>Отчётность</t>
+          <t>Подстрим 5.7</t>
         </is>
       </c>
       <c r="C9" s="70" t="n"/>
@@ -8059,7 +8094,7 @@
       <c r="A10" s="70" t="n"/>
       <c r="B10" s="70" t="inlineStr">
         <is>
-          <t>Регламенты</t>
+          <t>Подстрим 5.8</t>
         </is>
       </c>
       <c r="C10" s="70" t="n"/>

</xml_diff>